<commit_message>
Expand StemIndexer sequence length cases
</commit_message>
<xml_diff>
--- a/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
+++ b/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1faa11aeb4554a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2b57a2d1a1384fa8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -553,13 +553,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G2" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[3968]</x:v>
       </x:c>
       <x:c r="H2" s="17" t="str">
-        <x:v>[2048]</x:v>
+        <x:v>[7296]</x:v>
       </x:c>
       <x:c r="I2" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[3968]</x:v>
       </x:c>
       <x:c r="J2" s="18" t="b">
         <x:v>1</x:v>
@@ -1153,13 +1153,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G12" s="17" t="str">
-        <x:v>[2048]</x:v>
+        <x:v>[7296]</x:v>
       </x:c>
       <x:c r="H12" s="17" t="str">
-        <x:v>[4096]</x:v>
+        <x:v>[32768]</x:v>
       </x:c>
       <x:c r="I12" s="17" t="str">
-        <x:v>[2048]</x:v>
+        <x:v>[7296]</x:v>
       </x:c>
       <x:c r="J12" s="18" t="b">
         <x:v>1</x:v>
@@ -2293,13 +2293,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G31" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[32768]</x:v>
       </x:c>
       <x:c r="H31" s="17" t="str">
-        <x:v>[4096]</x:v>
+        <x:v>[7296]</x:v>
       </x:c>
       <x:c r="I31" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[7296]</x:v>
       </x:c>
       <x:c r="J31" s="18" t="b">
         <x:v>0</x:v>
@@ -2355,13 +2355,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G32" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[262144]</x:v>
       </x:c>
       <x:c r="H32" s="17" t="str">
-        <x:v>[4096]</x:v>
+        <x:v>[128]</x:v>
       </x:c>
       <x:c r="I32" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[128]</x:v>
       </x:c>
       <x:c r="J32" s="18" t="b">
         <x:v>0</x:v>
@@ -2522,7 +2522,7 @@
         <x:v>SI_WB_034</x:v>
       </x:c>
       <x:c r="B35" s="17" t="str">
-        <x:v>decode_causal_s2_two_loop_tail</x:v>
+        <x:v>decode_causal_s2_8192_blocks</x:v>
       </x:c>
       <x:c r="C35" s="17" t="str">
         <x:v>PASS</x:v>
@@ -2540,10 +2540,10 @@
         <x:v>[1]</x:v>
       </x:c>
       <x:c r="H35" s="17" t="str">
-        <x:v>[33409]</x:v>
+        <x:v>[1048576]</x:v>
       </x:c>
       <x:c r="I35" s="17" t="str">
-        <x:v>[33408]</x:v>
+        <x:v>[1048575]</x:v>
       </x:c>
       <x:c r="J35" s="18" t="b">
         <x:v>1</x:v>
@@ -2574,7 +2574,7 @@
       </x:c>
       <x:c r="S35" s="17" t="str"/>
       <x:c r="T35" s="19" t="str">
-        <x:v>SI_WB_034 decode_causal_s2_two_loop_tail 覆盖: decode；causal；S1=1；S2跨两个基本块并带尾块 设计: 单token decode下保持较长KV，验证causal有效S2和多S2 loop合并。</x:v>
+        <x:v>SI_WB_034 decode_causal_s2_8192_blocks 覆盖: decode；causal；S1=1；S2达到8192个block 设计: 单token decode下保持超长KV，验证causal有效S2和多S2 loop合并。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
@@ -3062,7 +3062,7 @@
         <x:v>SI_WB_043</x:v>
       </x:c>
       <x:c r="B44" s="17" t="str">
-        <x:v>gqa_q64_kv2_noncausal_s2_tail</x:v>
+        <x:v>gqa_q64_kv2_noncausal_s2_2048_blocks</x:v>
       </x:c>
       <x:c r="C44" s="17" t="str">
         <x:v>PASS</x:v>
@@ -3077,13 +3077,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G44" s="17" t="str">
-        <x:v>[512]</x:v>
+        <x:v>[128]</x:v>
       </x:c>
       <x:c r="H44" s="17" t="str">
-        <x:v>[33408]</x:v>
+        <x:v>[262144]</x:v>
       </x:c>
       <x:c r="I44" s="17" t="str">
-        <x:v>[512]</x:v>
+        <x:v>[128]</x:v>
       </x:c>
       <x:c r="J44" s="18" t="b">
         <x:v>0</x:v>
@@ -3114,7 +3114,7 @@
       </x:c>
       <x:c r="S44" s="17" t="str"/>
       <x:c r="T44" s="19" t="str">
-        <x:v>SI_WB_043 gqa_q64_kv2_noncausal_s2_tail 覆盖: q_heads=64；kv_heads=2；g=32；non-causal；S2多loop尾块 设计: 组合大G和长S2尾块，验证GQA映射和ProcessTopK多S2合并。</x:v>
+        <x:v>SI_WB_043 gqa_q64_kv2_noncausal_s2_2048_blocks 覆盖: q_heads=64；kv_heads=2；g=32；non-causal；S2达到2048个block 设计: 组合大G和长S2，验证GQA映射和ProcessTopK多S2合并。</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
@@ -3962,13 +3962,13 @@
         <x:v>SI_WB_058</x:v>
       </x:c>
       <x:c r="B59" s="17" t="str">
-        <x:v>batch20_decode_q64_kv2_prompt_tail</x:v>
+        <x:v>decode_q64_kv2_16k_blocks</x:v>
       </x:c>
       <x:c r="C59" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D59" s="17" t="n">
-        <x:v>20</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E59" s="17" t="n">
         <x:v>64</x:v>
@@ -3977,13 +3977,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G59" s="17" t="str">
-        <x:v>[1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1]</x:v>
+        <x:v>[1]</x:v>
       </x:c>
       <x:c r="H59" s="17" t="str">
-        <x:v>[12289,12290,12291,12292,12293,12294,12295,12296,12297,12298,12299,12300,12301,12302,12303,12304,12305,12306,12307,12308]</x:v>
+        <x:v>[2097152]</x:v>
       </x:c>
       <x:c r="I59" s="17" t="str">
-        <x:v>[12288,12289,12290,12291,12292,12293,12294,12295,12296,12297,12298,12299,12300,12301,12302,12303,12304,12305,12306,12307]</x:v>
+        <x:v>[2097151]</x:v>
       </x:c>
       <x:c r="J59" s="18" t="b">
         <x:v>1</x:v>
@@ -4014,7 +4014,7 @@
       </x:c>
       <x:c r="S59" s="17" t="str"/>
       <x:c r="T59" s="19" t="str">
-        <x:v>SI_WB_058 batch20_decode_q64_kv2_prompt_tail 覆盖: batch=20；q64/kv2；decode；长KV尾块 设计: 大G decode路径下，验证prompt长度与kv长度错开一位时的metadata和golden对齐。</x:v>
+        <x:v>SI_WB_058 decode_q64_kv2_16k_blocks 覆盖: batch=1；q64/kv2；decode；KV长度达到16384个block 设计: 大G decode路径下覆盖超长KV，验证prompt长度与kv长度错开一位时的metadata和golden对齐。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
@@ -4140,7 +4140,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ce836bfdf1d4cae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b0aec76748849ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine StemIndexer long sequence pytest cases
</commit_message>
<xml_diff>
--- a/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
+++ b/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2b57a2d1a1384fa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb0a55a25dabb42ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -538,7 +538,7 @@
         <x:v>SI_WB_001</x:v>
       </x:c>
       <x:c r="B2" s="17" t="str">
-        <x:v>basic_prefill_small_prompt_no_tail</x:v>
+        <x:v>basic_prefill_32k_kv_no_tail</x:v>
       </x:c>
       <x:c r="C2" s="17" t="str">
         <x:v>PASS</x:v>
@@ -556,10 +556,10 @@
         <x:v>[3968]</x:v>
       </x:c>
       <x:c r="H2" s="17" t="str">
-        <x:v>[7296]</x:v>
+        <x:v>[32768]</x:v>
       </x:c>
       <x:c r="I2" s="17" t="str">
-        <x:v>[3968]</x:v>
+        <x:v>[32768]</x:v>
       </x:c>
       <x:c r="J2" s="18" t="b">
         <x:v>1</x:v>
@@ -590,7 +590,7 @@
       </x:c>
       <x:c r="S2" s="17" t="str"/>
       <x:c r="T2" s="19" t="str">
-        <x:v>SI_WB_001 basic_prefill_small_prompt_no_tail 覆盖: 基础链路；prefill；small prompt分支；q/kv无尾块；causal=true 设计: 所有固定规格使用合法默认值，先验证 StemIndexer 端到端最基础路径。</x:v>
+        <x:v>SI_WB_001 basic_prefill_32k_kv_no_tail 覆盖: 基础链路；prefill；kv/prompt为32K token；causal=true 设计: query长度保持原基础case，只把KV和prompt拉到32K token基准线。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -1156,10 +1156,10 @@
         <x:v>[7296]</x:v>
       </x:c>
       <x:c r="H12" s="17" t="str">
-        <x:v>[32768]</x:v>
+        <x:v>[65536]</x:v>
       </x:c>
       <x:c r="I12" s="17" t="str">
-        <x:v>[7296]</x:v>
+        <x:v>[65536]</x:v>
       </x:c>
       <x:c r="J12" s="18" t="b">
         <x:v>1</x:v>
@@ -1216,10 +1216,10 @@
         <x:v>[8192]</x:v>
       </x:c>
       <x:c r="H13" s="17" t="str">
-        <x:v>[8192]</x:v>
+        <x:v>[32768]</x:v>
       </x:c>
       <x:c r="I13" s="17" t="str">
-        <x:v>[8192]</x:v>
+        <x:v>[32768]</x:v>
       </x:c>
       <x:c r="J13" s="18" t="b">
         <x:v>1</x:v>
@@ -1250,7 +1250,7 @@
       </x:c>
       <x:c r="S13" s="17" t="str"/>
       <x:c r="T13" s="19" t="str">
-        <x:v>SI_WB_012 alpha_decay_half 覆盖: TPD alpha=0.5；后部query预算下降 设计: 覆盖普通衰减路径，golden 应检查后部 query block 的 k(i) 小于前部。</x:v>
+        <x:v>SI_WB_012 alpha_decay_half 覆盖: TPD alpha=0.5；后部query预算下降；kv/prompt为32K token 设计: query长度保持不变，在32K KV/prompt基准线上覆盖普通衰减路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1276,10 +1276,10 @@
         <x:v>[8192]</x:v>
       </x:c>
       <x:c r="H14" s="17" t="str">
-        <x:v>[8192]</x:v>
+        <x:v>[65536]</x:v>
       </x:c>
       <x:c r="I14" s="17" t="str">
-        <x:v>[8192]</x:v>
+        <x:v>[65536]</x:v>
       </x:c>
       <x:c r="J14" s="18" t="b">
         <x:v>1</x:v>
@@ -1310,7 +1310,7 @@
       </x:c>
       <x:c r="S14" s="17" t="str"/>
       <x:c r="T14" s="19" t="str">
-        <x:v>SI_WB_013 alpha_small_positive 覆盖: alpha接近合法下界；强衰减；topkCurr clamp 设计: alpha 接近 0 但仍合法，覆盖预算强衰减以及 topkCurr 与 s2Valid 的 clamp。</x:v>
+        <x:v>SI_WB_013 alpha_small_positive 覆盖: alpha接近合法下界；强衰减；topkCurr clamp；kv/prompt为64K token 设计: query长度保持不变，在64K KV/prompt基准线上覆盖预算强衰减。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -2218,7 +2218,7 @@
         <x:v>SI_WB_029</x:v>
       </x:c>
       <x:c r="B30" s="17" t="str">
-        <x:v>decode_single_token_long_kv</x:v>
+        <x:v>decode_single_token_64k_kv</x:v>
       </x:c>
       <x:c r="C30" s="17" t="str">
         <x:v>PASS</x:v>
@@ -2236,10 +2236,10 @@
         <x:v>[1]</x:v>
       </x:c>
       <x:c r="H30" s="17" t="str">
-        <x:v>[8193]</x:v>
+        <x:v>[65536]</x:v>
       </x:c>
       <x:c r="I30" s="17" t="str">
-        <x:v>[8192]</x:v>
+        <x:v>[65535]</x:v>
       </x:c>
       <x:c r="J30" s="18" t="b">
         <x:v>1</x:v>
@@ -2270,7 +2270,7 @@
       </x:c>
       <x:c r="S30" s="17" t="str"/>
       <x:c r="T30" s="19" t="str">
-        <x:v>SI_WB_029 decode_single_token_long_kv 覆盖: decode路径；q_len=1；kv_len参与i/N；kv尾块 设计: 单 token decode 是设计方案明确风险点，预算应按 kv_len 而不是 q_len 计算。</x:v>
+        <x:v>SI_WB_029 decode_single_token_64k_kv 覆盖: decode路径；q_len=1；kv_len=64K；kv_len参与i/N 设计: 单 token decode 是设计方案明确风险点，预算应按 kv_len 而不是 q_len 计算。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
@@ -2402,7 +2402,7 @@
         <x:v>SI_WB_032</x:v>
       </x:c>
       <x:c r="B33" s="17" t="str">
-        <x:v>dynamic_topk_large_prompt_decode</x:v>
+        <x:v>dynamic_topk_128k_prompt_decode</x:v>
       </x:c>
       <x:c r="C33" s="17" t="str">
         <x:v>PASS</x:v>
@@ -2420,10 +2420,10 @@
         <x:v>[1]</x:v>
       </x:c>
       <x:c r="H33" s="17" t="str">
-        <x:v>[20481]</x:v>
+        <x:v>[131073]</x:v>
       </x:c>
       <x:c r="I33" s="17" t="str">
-        <x:v>[20480]</x:v>
+        <x:v>[131072]</x:v>
       </x:c>
       <x:c r="J33" s="18" t="b">
         <x:v>1</x:v>
@@ -2454,7 +2454,7 @@
       </x:c>
       <x:c r="S33" s="17" t="str"/>
       <x:c r="T33" s="19" t="str">
-        <x:v>SI_WB_032 dynamic_topk_large_prompt_decode 覆盖: num_prompt_tokens=20480；prompt block=160；large分支；decode路径下alpha衰减 设计: 当前TopK预算按prompt block数分段，构造单token decode降低计算量并覆盖large分支。</x:v>
+        <x:v>SI_WB_032 dynamic_topk_128k_prompt_decode 覆盖: num_prompt_tokens=128K；prompt block=1024；large分支；decode路径下alpha衰减 设计: query长度保持单token decode，以128K prompt覆盖large分支下的长上下文预算计算。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
@@ -2582,7 +2582,7 @@
         <x:v>SI_WB_035</x:v>
       </x:c>
       <x:c r="B36" s="17" t="str">
-        <x:v>decode_prompt_not_divisible</x:v>
+        <x:v>decode_prompt_128k_not_divisible</x:v>
       </x:c>
       <x:c r="C36" s="17" t="str">
         <x:v>PASS</x:v>
@@ -2600,10 +2600,10 @@
         <x:v>[1]</x:v>
       </x:c>
       <x:c r="H36" s="17" t="str">
-        <x:v>[8194]</x:v>
+        <x:v>[131072]</x:v>
       </x:c>
       <x:c r="I36" s="17" t="str">
-        <x:v>[8193]</x:v>
+        <x:v>[131071]</x:v>
       </x:c>
       <x:c r="J36" s="18" t="b">
         <x:v>1</x:v>
@@ -2634,7 +2634,7 @@
       </x:c>
       <x:c r="S36" s="17" t="str"/>
       <x:c r="T36" s="19" t="str">
-        <x:v>SI_WB_035 decode_prompt_not_divisible 覆盖: decode；num_prompt_tokens非128整数倍；prompt block向上取整 设计: num_prompt_tokens=8193，验证promptLen=ceil(8193/128)路径。</x:v>
+        <x:v>SI_WB_035 decode_prompt_128k_not_divisible 覆盖: decode；num_prompt_tokens非128整数倍；prompt block向上取整 设计: num_prompt_tokens=131071，验证128K附近promptLen向上取整路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -2814,7 +2814,7 @@
       </x:c>
       <x:c r="S39" s="17" t="str"/>
       <x:c r="T39" s="19" t="str">
-        <x:v>SI_WB_038 dynamic_topk_medium_upper_159 覆盖: 动态TopK medium分支上边界；numPromptK=159 设计: prompt block数刚好小于160，验证medium分支高位边界。</x:v>
+        <x:v>SI_WB_038 dynamic_topk_medium_upper_159 覆盖: 动态TopK medium分支上边界；numPromptK=159；kv为32K token 设计: query长度保持不变，以32K KV覆盖medium分支高位边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
@@ -2874,7 +2874,7 @@
       </x:c>
       <x:c r="S40" s="17" t="str"/>
       <x:c r="T40" s="19" t="str">
-        <x:v>SI_WB_039 dynamic_topk_large_lower_160 覆盖: 动态TopK large分支下边界；numPromptK=160 设计: prompt block数等于160，验证从medium切到large的分段点。</x:v>
+        <x:v>SI_WB_039 dynamic_topk_large_lower_160 覆盖: 动态TopK large分支下边界；numPromptK=160；kv为32K token 设计: query长度保持不变，以32K KV覆盖从medium切到large的分段点。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
@@ -4140,7 +4140,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b0aec76748849ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5de71e7fd3543cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine StemIndexer pytest prompt cases
</commit_message>
<xml_diff>
--- a/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
+++ b/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb0a55a25dabb42ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R9c1718c6bb544f4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -227,7 +227,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StemIndexerCases" displayName="StemIndexerCases" ref="A1:T61" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StemIndexerCases" displayName="StemIndexerCases" ref="A1:T58" headerRowCount="1">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="case_id"/>
     <x:tableColumn id="2" name="testcase_name"/>
@@ -619,7 +619,7 @@
         <x:v>[2048]</x:v>
       </x:c>
       <x:c r="I3" s="17" t="str">
-        <x:v>[1153]</x:v>
+        <x:v>[2048]</x:v>
       </x:c>
       <x:c r="J3" s="18" t="b">
         <x:v>1</x:v>
@@ -679,7 +679,7 @@
         <x:v>[2305]</x:v>
       </x:c>
       <x:c r="I4" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[2305]</x:v>
       </x:c>
       <x:c r="J4" s="18" t="b">
         <x:v>1</x:v>
@@ -739,7 +739,7 @@
         <x:v>[257,513,769,1025,1281,1537,1793]</x:v>
       </x:c>
       <x:c r="I5" s="17" t="str">
-        <x:v>[129,257,385,513,641,769,897]</x:v>
+        <x:v>[257,513,769,1025,1281,1537,1793]</x:v>
       </x:c>
       <x:c r="J5" s="18" t="b">
         <x:v>1</x:v>
@@ -859,7 +859,7 @@
         <x:v>[896,1024,1152,1280,1408]</x:v>
       </x:c>
       <x:c r="I7" s="17" t="str">
-        <x:v>[640,768,896,1024,1152]</x:v>
+        <x:v>[896,1024,1152,1280,1408]</x:v>
       </x:c>
       <x:c r="J7" s="18" t="b">
         <x:v>0</x:v>
@@ -919,7 +919,7 @@
         <x:v>[2048,2305,2561,2817,3073,3329,3585,3841,4097,4353,4609]</x:v>
       </x:c>
       <x:c r="I8" s="17" t="str">
-        <x:v>[512,640,769,896,1025,1153,1281,1409,1537,1665,1793]</x:v>
+        <x:v>[2048,2305,2561,2817,3073,3329,3585,3841,4097,4353,4609]</x:v>
       </x:c>
       <x:c r="J8" s="18" t="b">
         <x:v>0</x:v>
@@ -979,7 +979,7 @@
         <x:v>[256,256,256,256,256,256,256,256,256,256]</x:v>
       </x:c>
       <x:c r="I9" s="17" t="str">
-        <x:v>[128,129,130,160,192,224,225,240,248,256]</x:v>
+        <x:v>[256,256,256,256,256,256,256,256,256,256]</x:v>
       </x:c>
       <x:c r="J9" s="18" t="b">
         <x:v>0</x:v>
@@ -1039,7 +1039,7 @@
         <x:v>[4096]</x:v>
       </x:c>
       <x:c r="I10" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[4096]</x:v>
       </x:c>
       <x:c r="J10" s="18" t="b">
         <x:v>1</x:v>
@@ -1099,7 +1099,7 @@
         <x:v>[4096,4353,4609,4865,5121,5377]</x:v>
       </x:c>
       <x:c r="I11" s="17" t="str">
-        <x:v>[1024,1152,1280,1408,1536,1664]</x:v>
+        <x:v>[4096,4353,4609,4865,5121,5377]</x:v>
       </x:c>
       <x:c r="J11" s="18" t="b">
         <x:v>0</x:v>
@@ -1339,7 +1339,7 @@
         <x:v>[16384,16384]</x:v>
       </x:c>
       <x:c r="I15" s="17" t="str">
-        <x:v>[512,1024]</x:v>
+        <x:v>[16384,16384]</x:v>
       </x:c>
       <x:c r="J15" s="18" t="b">
         <x:v>1</x:v>
@@ -1399,7 +1399,7 @@
         <x:v>[16385,16385]</x:v>
       </x:c>
       <x:c r="I16" s="17" t="str">
-        <x:v>[512,1024]</x:v>
+        <x:v>[16385,16385]</x:v>
       </x:c>
       <x:c r="J16" s="18" t="b">
         <x:v>1</x:v>
@@ -1459,7 +1459,7 @@
         <x:v>[32768,32768]</x:v>
       </x:c>
       <x:c r="I17" s="17" t="str">
-        <x:v>[512,1024]</x:v>
+        <x:v>[32768,32768]</x:v>
       </x:c>
       <x:c r="J17" s="18" t="b">
         <x:v>1</x:v>
@@ -1519,7 +1519,7 @@
         <x:v>[32769,32769]</x:v>
       </x:c>
       <x:c r="I18" s="17" t="str">
-        <x:v>[512,1024]</x:v>
+        <x:v>[32769,32769]</x:v>
       </x:c>
       <x:c r="J18" s="18" t="b">
         <x:v>1</x:v>
@@ -1579,7 +1579,7 @@
         <x:v>[4096]</x:v>
       </x:c>
       <x:c r="I19" s="17" t="str">
-        <x:v>[3072]</x:v>
+        <x:v>[4096]</x:v>
       </x:c>
       <x:c r="J19" s="18" t="b">
         <x:v>1</x:v>
@@ -1639,7 +1639,7 @@
         <x:v>[4096]</x:v>
       </x:c>
       <x:c r="I20" s="17" t="str">
-        <x:v>[3200]</x:v>
+        <x:v>[4096]</x:v>
       </x:c>
       <x:c r="J20" s="18" t="b">
         <x:v>1</x:v>
@@ -1699,7 +1699,7 @@
         <x:v>[4096]</x:v>
       </x:c>
       <x:c r="I21" s="17" t="str">
-        <x:v>[384]</x:v>
+        <x:v>[4096]</x:v>
       </x:c>
       <x:c r="J21" s="18" t="b">
         <x:v>1</x:v>
@@ -1759,7 +1759,7 @@
         <x:v>[4096]</x:v>
       </x:c>
       <x:c r="I22" s="17" t="str">
-        <x:v>[512]</x:v>
+        <x:v>[4096]</x:v>
       </x:c>
       <x:c r="J22" s="18" t="b">
         <x:v>1</x:v>
@@ -1819,7 +1819,7 @@
         <x:v>[2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608,4864,5120]</x:v>
       </x:c>
       <x:c r="I23" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048]</x:v>
+        <x:v>[2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608,4864,5120]</x:v>
       </x:c>
       <x:c r="J23" s="18" t="b">
         <x:v>1</x:v>
@@ -1879,7 +1879,7 @@
         <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352]</x:v>
       </x:c>
       <x:c r="I24" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176]</x:v>
+        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352]</x:v>
       </x:c>
       <x:c r="J24" s="18" t="b">
         <x:v>1</x:v>
@@ -1939,7 +1939,7 @@
         <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072]</x:v>
       </x:c>
       <x:c r="I25" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536]</x:v>
+        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072]</x:v>
       </x:c>
       <x:c r="J25" s="18" t="b">
         <x:v>1</x:v>
@@ -1999,7 +1999,7 @@
         <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608]</x:v>
       </x:c>
       <x:c r="I26" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304]</x:v>
+        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608]</x:v>
       </x:c>
       <x:c r="J26" s="18" t="b">
         <x:v>1</x:v>
@@ -2059,7 +2059,7 @@
         <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608,4864]</x:v>
       </x:c>
       <x:c r="I27" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304,2432]</x:v>
+        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608,4864]</x:v>
       </x:c>
       <x:c r="J27" s="18" t="b">
         <x:v>1</x:v>
@@ -2119,7 +2119,7 @@
         <x:v>[512,768,1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608]</x:v>
       </x:c>
       <x:c r="I28" s="17" t="str">
-        <x:v>[256,384,512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304]</x:v>
+        <x:v>[512,768,1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608]</x:v>
       </x:c>
       <x:c r="J28" s="18" t="b">
         <x:v>1</x:v>
@@ -2179,7 +2179,7 @@
         <x:v>[1024,8193,1280,8194,1536,8195,1792,8196,2048,8197,2304,8198,2560,8199,2816,8200,3072,8201,3328]</x:v>
       </x:c>
       <x:c r="I29" s="17" t="str">
-        <x:v>[512,8192,640,8193,768,8194,896,8195,1024,8196,1152,8197,1280,8198,1408,8199,1536,8200,1664]</x:v>
+        <x:v>[1024,8193,1280,8194,1536,8195,1792,8196,2048,8197,2304,8198,2560,8199,2816,8200,3072,8201,3328]</x:v>
       </x:c>
       <x:c r="J29" s="18" t="b">
         <x:v>1</x:v>
@@ -2239,7 +2239,7 @@
         <x:v>[65536]</x:v>
       </x:c>
       <x:c r="I30" s="17" t="str">
-        <x:v>[65535]</x:v>
+        <x:v>[65536]</x:v>
       </x:c>
       <x:c r="J30" s="18" t="b">
         <x:v>1</x:v>
@@ -2355,7 +2355,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G32" s="17" t="str">
-        <x:v>[262144]</x:v>
+        <x:v>[1024]</x:v>
       </x:c>
       <x:c r="H32" s="17" t="str">
         <x:v>[128]</x:v>
@@ -2394,7 +2394,7 @@
         <x:v>qflat=constant_positive; kflat=constant_positive; vbias=zeros</x:v>
       </x:c>
       <x:c r="T32" s="19" t="str">
-        <x:v>SI_WB_031 score_scale_rs64 覆盖: scoreScale=1/64；DivRs路径；B/stride固定推导 设计: 固定规格 B=128、stride=16 推出 Rs=64，构造常量输入方便 golden 检查缩放方向和量级。</x:v>
+        <x:v>SI_WB_031 score_scale_rs64 覆盖: scoreScale=1/64；DivRs路径；B/stride固定推导 设计: 固定规格 B=128、stride=16 推出 Rs=64，用小Q和常量输入检查缩放方向和量级。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -2420,7 +2420,7 @@
         <x:v>[1]</x:v>
       </x:c>
       <x:c r="H33" s="17" t="str">
-        <x:v>[131073]</x:v>
+        <x:v>[131072]</x:v>
       </x:c>
       <x:c r="I33" s="17" t="str">
         <x:v>[131072]</x:v>
@@ -2483,7 +2483,7 @@
         <x:v>[33408]</x:v>
       </x:c>
       <x:c r="I34" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[33408]</x:v>
       </x:c>
       <x:c r="J34" s="18" t="b">
         <x:v>0</x:v>
@@ -2519,10 +2519,10 @@
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="16" t="str">
-        <x:v>SI_WB_034</x:v>
+        <x:v>SI_WB_035</x:v>
       </x:c>
       <x:c r="B35" s="17" t="str">
-        <x:v>decode_causal_s2_8192_blocks</x:v>
+        <x:v>decode_prompt_128k_not_divisible</x:v>
       </x:c>
       <x:c r="C35" s="17" t="str">
         <x:v>PASS</x:v>
@@ -2531,25 +2531,25 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E35" s="17" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F35" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G35" s="17" t="str">
         <x:v>[1]</x:v>
       </x:c>
       <x:c r="H35" s="17" t="str">
-        <x:v>[1048576]</x:v>
+        <x:v>[131071]</x:v>
       </x:c>
       <x:c r="I35" s="17" t="str">
-        <x:v>[1048575]</x:v>
+        <x:v>[131071]</x:v>
       </x:c>
       <x:c r="J35" s="18" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K35" s="17" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L35" s="17" t="n">
         <x:v>128</x:v>
@@ -2574,15 +2574,15 @@
       </x:c>
       <x:c r="S35" s="17" t="str"/>
       <x:c r="T35" s="19" t="str">
-        <x:v>SI_WB_034 decode_causal_s2_8192_blocks 覆盖: decode；causal；S1=1；S2达到8192个block 设计: 单token decode下保持超长KV，验证causal有效S2和多S2 loop合并。</x:v>
+        <x:v>SI_WB_035 decode_prompt_128k_not_divisible 覆盖: decode；num_prompt_tokens非128整数倍；prompt block向上取整 设计: num_prompt_tokens=131071，验证128K附近promptLen向上取整路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="16" t="str">
-        <x:v>SI_WB_035</x:v>
+        <x:v>SI_WB_036</x:v>
       </x:c>
       <x:c r="B36" s="17" t="str">
-        <x:v>decode_prompt_128k_not_divisible</x:v>
+        <x:v>dynamic_topk_small_upper_55</x:v>
       </x:c>
       <x:c r="C36" s="17" t="str">
         <x:v>PASS</x:v>
@@ -2594,19 +2594,19 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="F36" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G36" s="17" t="str">
-        <x:v>[1]</x:v>
+        <x:v>[1024]</x:v>
       </x:c>
       <x:c r="H36" s="17" t="str">
-        <x:v>[131072]</x:v>
+        <x:v>[7040]</x:v>
       </x:c>
       <x:c r="I36" s="17" t="str">
-        <x:v>[131071]</x:v>
+        <x:v>[7040]</x:v>
       </x:c>
       <x:c r="J36" s="18" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K36" s="17" t="n">
         <x:v>1</x:v>
@@ -2634,15 +2634,15 @@
       </x:c>
       <x:c r="S36" s="17" t="str"/>
       <x:c r="T36" s="19" t="str">
-        <x:v>SI_WB_035 decode_prompt_128k_not_divisible 覆盖: decode；num_prompt_tokens非128整数倍；prompt block向上取整 设计: num_prompt_tokens=131071，验证128K附近promptLen向上取整路径。</x:v>
+        <x:v>SI_WB_036 dynamic_topk_small_upper_55 覆盖: 动态TopK small分支上边界；numPromptK=55 设计: prompt block数刚好小于56，验证kStart=numPromptK的边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="16" t="str">
-        <x:v>SI_WB_036</x:v>
+        <x:v>SI_WB_037</x:v>
       </x:c>
       <x:c r="B37" s="17" t="str">
-        <x:v>dynamic_topk_small_upper_55</x:v>
+        <x:v>dynamic_topk_medium_lower_56</x:v>
       </x:c>
       <x:c r="C37" s="17" t="str">
         <x:v>PASS</x:v>
@@ -2651,19 +2651,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E37" s="17" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F37" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G37" s="17" t="str">
         <x:v>[1024]</x:v>
       </x:c>
       <x:c r="H37" s="17" t="str">
-        <x:v>[16384]</x:v>
+        <x:v>[7168]</x:v>
       </x:c>
       <x:c r="I37" s="17" t="str">
-        <x:v>[7040]</x:v>
+        <x:v>[7168]</x:v>
       </x:c>
       <x:c r="J37" s="18" t="b">
         <x:v>0</x:v>
@@ -2694,15 +2694,15 @@
       </x:c>
       <x:c r="S37" s="17" t="str"/>
       <x:c r="T37" s="19" t="str">
-        <x:v>SI_WB_036 dynamic_topk_small_upper_55 覆盖: 动态TopK small分支上边界；numPromptK=55 设计: prompt block数刚好小于56，验证kStart=numPromptK的边界。</x:v>
+        <x:v>SI_WB_037 dynamic_topk_medium_lower_56 覆盖: 动态TopK medium分支下边界；numPromptK=56 设计: prompt block数等于56，验证从small切到medium的分段点。</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="16" t="str">
-        <x:v>SI_WB_037</x:v>
+        <x:v>SI_WB_038</x:v>
       </x:c>
       <x:c r="B38" s="17" t="str">
-        <x:v>dynamic_topk_medium_lower_56</x:v>
+        <x:v>dynamic_topk_medium_upper_159</x:v>
       </x:c>
       <x:c r="C38" s="17" t="str">
         <x:v>PASS</x:v>
@@ -2711,25 +2711,25 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E38" s="17" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F38" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G38" s="17" t="str">
         <x:v>[1024]</x:v>
       </x:c>
       <x:c r="H38" s="17" t="str">
-        <x:v>[16384]</x:v>
+        <x:v>[20352]</x:v>
       </x:c>
       <x:c r="I38" s="17" t="str">
-        <x:v>[7168]</x:v>
+        <x:v>[20352]</x:v>
       </x:c>
       <x:c r="J38" s="18" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K38" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="L38" s="17" t="n">
         <x:v>128</x:v>
@@ -2754,15 +2754,15 @@
       </x:c>
       <x:c r="S38" s="17" t="str"/>
       <x:c r="T38" s="19" t="str">
-        <x:v>SI_WB_037 dynamic_topk_medium_lower_56 覆盖: 动态TopK medium分支下边界；numPromptK=56 设计: prompt block数等于56，验证从small切到medium的分段点。</x:v>
+        <x:v>SI_WB_038 dynamic_topk_medium_upper_159 覆盖: 动态TopK medium分支上边界；numPromptK=159；kv为32K token 设计: query长度保持不变，以32K KV覆盖medium分支高位边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="16" t="str">
-        <x:v>SI_WB_038</x:v>
+        <x:v>SI_WB_039</x:v>
       </x:c>
       <x:c r="B39" s="17" t="str">
-        <x:v>dynamic_topk_medium_upper_159</x:v>
+        <x:v>dynamic_topk_large_lower_160</x:v>
       </x:c>
       <x:c r="C39" s="17" t="str">
         <x:v>PASS</x:v>
@@ -2774,22 +2774,22 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="F39" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G39" s="17" t="str">
         <x:v>[1024]</x:v>
       </x:c>
       <x:c r="H39" s="17" t="str">
-        <x:v>[32768]</x:v>
+        <x:v>[20480]</x:v>
       </x:c>
       <x:c r="I39" s="17" t="str">
-        <x:v>[20352]</x:v>
+        <x:v>[20480]</x:v>
       </x:c>
       <x:c r="J39" s="18" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K39" s="17" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="L39" s="17" t="n">
         <x:v>128</x:v>
@@ -2814,42 +2814,42 @@
       </x:c>
       <x:c r="S39" s="17" t="str"/>
       <x:c r="T39" s="19" t="str">
-        <x:v>SI_WB_038 dynamic_topk_medium_upper_159 覆盖: 动态TopK medium分支上边界；numPromptK=159；kv为32K token 设计: query长度保持不变，以32K KV覆盖medium分支高位边界。</x:v>
+        <x:v>SI_WB_039 dynamic_topk_large_lower_160 覆盖: 动态TopK large分支下边界；numPromptK=160；kv为32K token 设计: query长度保持不变，以32K KV覆盖从medium切到large的分段点。</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="16" t="str">
-        <x:v>SI_WB_039</x:v>
+        <x:v>SI_WB_040</x:v>
       </x:c>
       <x:c r="B40" s="17" t="str">
-        <x:v>dynamic_topk_large_lower_160</x:v>
+        <x:v>batch12_mixed_prefill_decode</x:v>
       </x:c>
       <x:c r="C40" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D40" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E40" s="17" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="F40" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G40" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[128,513,1,640,1,768,1,896,1,1024,1,1152]</x:v>
       </x:c>
       <x:c r="H40" s="17" t="str">
-        <x:v>[32768]</x:v>
+        <x:v>[512,1025,8194,1280,8195,1536,8196,1792,8197,2048,8198,2304]</x:v>
       </x:c>
       <x:c r="I40" s="17" t="str">
-        <x:v>[20480]</x:v>
+        <x:v>[512,1025,8194,1280,8195,1536,8196,1792,8197,2048,8198,2304]</x:v>
       </x:c>
       <x:c r="J40" s="18" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K40" s="17" t="n">
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L40" s="17" t="n">
         <x:v>128</x:v>
@@ -2874,36 +2874,36 @@
       </x:c>
       <x:c r="S40" s="17" t="str"/>
       <x:c r="T40" s="19" t="str">
-        <x:v>SI_WB_039 dynamic_topk_large_lower_160 覆盖: 动态TopK large分支下边界；numPromptK=160；kv为32K token 设计: query长度保持不变，以32K KV覆盖从medium切到large的分段点。</x:v>
+        <x:v>SI_WB_040 batch12_mixed_prefill_decode 覆盖: batch=12；prefill/decode混合；多batch不同q/kv尾块 设计: 同一case内混合短prompt、q尾块、decode和kv尾块，验证batch维读取。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="16" t="str">
-        <x:v>SI_WB_040</x:v>
+        <x:v>SI_WB_041</x:v>
       </x:c>
       <x:c r="B41" s="17" t="str">
-        <x:v>batch12_mixed_prefill_decode</x:v>
+        <x:v>causal_s1_s2_unequal_batch3_g16</x:v>
       </x:c>
       <x:c r="C41" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D41" s="17" t="n">
-        <x:v>12</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E41" s="17" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="F41" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G41" s="17" t="str">
-        <x:v>[128,513,1,640,1,768,1,896,1,1024,1,1152]</x:v>
+        <x:v>[768,1153,1537]</x:v>
       </x:c>
       <x:c r="H41" s="17" t="str">
-        <x:v>[512,1025,8194,1280,8195,1536,8196,1792,8197,2048,8198,2304]</x:v>
+        <x:v>[1793,2305,2817]</x:v>
       </x:c>
       <x:c r="I41" s="17" t="str">
-        <x:v>[128,513,8193,640,8194,768,8195,896,8196,1024,8197,1152]</x:v>
+        <x:v>[1793,2305,2817]</x:v>
       </x:c>
       <x:c r="J41" s="18" t="b">
         <x:v>1</x:v>
@@ -2934,21 +2934,21 @@
       </x:c>
       <x:c r="S41" s="17" t="str"/>
       <x:c r="T41" s="19" t="str">
-        <x:v>SI_WB_040 batch12_mixed_prefill_decode 覆盖: batch=12；prefill/decode混合；多batch不同q/kv尾块 设计: 同一case内混合短prompt、q尾块、decode和kv尾块，验证batch维读取。</x:v>
+        <x:v>SI_WB_041 causal_s1_s2_unequal_batch3_g16 覆盖: causal下S1/S2不相等；kbOffset参与dynamicTopK位置计算 设计: actS1=3、actS2=7，验证s1Pos和可见S2的偏移逻辑。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="16" t="str">
-        <x:v>SI_WB_041</x:v>
+        <x:v>SI_WB_042</x:v>
       </x:c>
       <x:c r="B42" s="17" t="str">
-        <x:v>causal_s1_s2_unequal_batch3_g16</x:v>
+        <x:v>causal_q_tail_s1_s2_batch5</x:v>
       </x:c>
       <x:c r="C42" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D42" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E42" s="17" t="n">
         <x:v>64</x:v>
@@ -2957,13 +2957,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G42" s="17" t="str">
-        <x:v>[768,1153,1537]</x:v>
+        <x:v>[641,769,897,1025,1153]</x:v>
       </x:c>
       <x:c r="H42" s="17" t="str">
-        <x:v>[1793,2305,2817]</x:v>
+        <x:v>[1537,1793,2049,2305,2561]</x:v>
       </x:c>
       <x:c r="I42" s="17" t="str">
-        <x:v>[768,1153,1537]</x:v>
+        <x:v>[1537,1793,2049,2305,2561]</x:v>
       </x:c>
       <x:c r="J42" s="18" t="b">
         <x:v>1</x:v>
@@ -2994,39 +2994,39 @@
       </x:c>
       <x:c r="S42" s="17" t="str"/>
       <x:c r="T42" s="19" t="str">
-        <x:v>SI_WB_041 causal_s1_s2_unequal_batch3_g16 覆盖: causal下S1/S2不相等；kbOffset参与dynamicTopK位置计算 设计: actS1=3、actS2=7，验证s1Pos和可见S2的偏移逻辑。</x:v>
+        <x:v>SI_WB_042 causal_q_tail_s1_s2_batch5 覆盖: causal；q尾块；S1/S2偏移；最后S1块可见范围变化 设计: q=385导致actS1=4，kv=1153导致actS2=10，同时覆盖尾块和因果偏移。</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="16" t="str">
-        <x:v>SI_WB_042</x:v>
+        <x:v>SI_WB_043</x:v>
       </x:c>
       <x:c r="B43" s="17" t="str">
-        <x:v>causal_q_tail_s1_s2_batch5</x:v>
+        <x:v>gqa_q64_kv2_noncausal_s2_2048_blocks</x:v>
       </x:c>
       <x:c r="C43" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D43" s="17" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E43" s="17" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="F43" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G43" s="17" t="str">
-        <x:v>[641,769,897,1025,1153]</x:v>
+        <x:v>[128]</x:v>
       </x:c>
       <x:c r="H43" s="17" t="str">
-        <x:v>[1537,1793,2049,2305,2561]</x:v>
+        <x:v>[262144]</x:v>
       </x:c>
       <x:c r="I43" s="17" t="str">
-        <x:v>[641,769,897,1025,1153]</x:v>
+        <x:v>[262144]</x:v>
       </x:c>
       <x:c r="J43" s="18" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K43" s="17" t="n">
         <x:v>1</x:v>
@@ -3054,15 +3054,15 @@
       </x:c>
       <x:c r="S43" s="17" t="str"/>
       <x:c r="T43" s="19" t="str">
-        <x:v>SI_WB_042 causal_q_tail_s1_s2_batch5 覆盖: causal；q尾块；S1/S2偏移；最后S1块可见范围变化 设计: q=385导致actS1=4，kv=1153导致actS2=10，同时覆盖尾块和因果偏移。</x:v>
+        <x:v>SI_WB_043 gqa_q64_kv2_noncausal_s2_2048_blocks 覆盖: q_heads=64；kv_heads=2；g=32；non-causal；S2达到2048个block 设计: 组合大G和长S2，验证GQA映射和ProcessTopK多S2合并。</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="16" t="str">
-        <x:v>SI_WB_043</x:v>
+        <x:v>SI_WB_044</x:v>
       </x:c>
       <x:c r="B44" s="17" t="str">
-        <x:v>gqa_q64_kv2_noncausal_s2_2048_blocks</x:v>
+        <x:v>gqa_q64_kv8_m_tail</x:v>
       </x:c>
       <x:c r="C44" s="17" t="str">
         <x:v>PASS</x:v>
@@ -3074,19 +3074,19 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="F44" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G44" s="17" t="str">
-        <x:v>[128]</x:v>
+        <x:v>[1664]</x:v>
       </x:c>
       <x:c r="H44" s="17" t="str">
-        <x:v>[262144]</x:v>
+        <x:v>[4096]</x:v>
       </x:c>
       <x:c r="I44" s="17" t="str">
-        <x:v>[128]</x:v>
+        <x:v>[4096]</x:v>
       </x:c>
       <x:c r="J44" s="18" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K44" s="17" t="n">
         <x:v>1</x:v>
@@ -3114,39 +3114,39 @@
       </x:c>
       <x:c r="S44" s="17" t="str"/>
       <x:c r="T44" s="19" t="str">
-        <x:v>SI_WB_043 gqa_q64_kv2_noncausal_s2_2048_blocks 覆盖: q_heads=64；kv_heads=2；g=32；non-causal；S2达到2048个block 设计: 组合大G和长S2，验证GQA映射和ProcessTopK多S2合并。</x:v>
+        <x:v>SI_WB_044 gqa_q64_kv8_m_tail 覆盖: q_heads=64；kv_heads=8；g=8；M方向尾块 设计: actS1=13时actS1*g=104，覆盖mBase=96后的尾块处理。</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="16" t="str">
-        <x:v>SI_WB_044</x:v>
+        <x:v>SI_WB_045</x:v>
       </x:c>
       <x:c r="B45" s="17" t="str">
-        <x:v>gqa_q64_kv8_m_tail</x:v>
+        <x:v>short2_total_output_equal_batch4</x:v>
       </x:c>
       <x:c r="C45" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D45" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E45" s="17" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F45" s="17" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="G45" s="17" t="str">
-        <x:v>[1664]</x:v>
+        <x:v>[512,512,512,512]</x:v>
       </x:c>
       <x:c r="H45" s="17" t="str">
-        <x:v>[4096]</x:v>
+        <x:v>[8320,8320,8320,8320]</x:v>
       </x:c>
       <x:c r="I45" s="17" t="str">
-        <x:v>[1664]</x:v>
+        <x:v>[17280,17280,17280,17280]</x:v>
       </x:c>
       <x:c r="J45" s="18" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K45" s="17" t="n">
         <x:v>1</x:v>
@@ -3174,15 +3174,15 @@
       </x:c>
       <x:c r="S45" s="17" t="str"/>
       <x:c r="T45" s="19" t="str">
-        <x:v>SI_WB_044 gqa_q64_kv8_m_tail 覆盖: q_heads=64；kv_heads=8；g=8；M方向尾块 设计: actS1=13时actS1*g=104，覆盖mBase=96后的尾块处理。</x:v>
+        <x:v>SI_WB_045 short2_total_output_equal_batch4 覆盖: 短路2边界；curS2Len == initial + dynamicTopK + window 设计: prompt block=135，dynamicTopK=57，totalOutput=65，kv block=65，应直接输出连续索引。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="16" t="str">
-        <x:v>SI_WB_045</x:v>
+        <x:v>SI_WB_046</x:v>
       </x:c>
       <x:c r="B46" s="17" t="str">
-        <x:v>short2_total_output_equal_batch4</x:v>
+        <x:v>short2_total_output_plus_one_batch4</x:v>
       </x:c>
       <x:c r="C46" s="17" t="str">
         <x:v>PASS</x:v>
@@ -3200,10 +3200,10 @@
         <x:v>[512,512,512,512]</x:v>
       </x:c>
       <x:c r="H46" s="17" t="str">
-        <x:v>[1536,1536,1536,1536]</x:v>
+        <x:v>[8448,8448,8448,8448]</x:v>
       </x:c>
       <x:c r="I46" s="17" t="str">
-        <x:v>[512,512,512,512]</x:v>
+        <x:v>[17280,17280,17280,17280]</x:v>
       </x:c>
       <x:c r="J46" s="18" t="b">
         <x:v>0</x:v>
@@ -3234,21 +3234,21 @@
       </x:c>
       <x:c r="S46" s="17" t="str"/>
       <x:c r="T46" s="19" t="str">
-        <x:v>SI_WB_045 short2_total_output_equal_batch4 覆盖: 短路2边界；curS2Len == initial + dynamicTopK + window 设计: prompt block=4，totalOutput=12，kv block=12，应直接输出连续索引。</x:v>
+        <x:v>SI_WB_046 short2_total_output_plus_one_batch4 覆盖: 短路2临界后一位；进入正常TopK路径 设计: prompt block=135，dynamicTopK=57，totalOutput=65，kv block=66，验证刚越过短路边界的行为。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="16" t="str">
-        <x:v>SI_WB_046</x:v>
+        <x:v>SI_WB_047</x:v>
       </x:c>
       <x:c r="B47" s="17" t="str">
-        <x:v>short2_total_output_plus_one_batch4</x:v>
+        <x:v>batch23_noncausal_varlen_q32_kv8</x:v>
       </x:c>
       <x:c r="C47" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D47" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E47" s="17" t="n">
         <x:v>32</x:v>
@@ -3257,13 +3257,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G47" s="17" t="str">
-        <x:v>[512,512,512,512]</x:v>
+        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304,2432,2560,2688,2816,2944,3072,3200,3328]</x:v>
       </x:c>
       <x:c r="H47" s="17" t="str">
-        <x:v>[1664,1664,1664,1664]</x:v>
+        <x:v>[4096,4352,4608,4864,5120,5376,5632,5888,6144,6400,6656,6912,7168,7424,7680,7936,8192,8448,8704,8960,9216,9472,9728]</x:v>
       </x:c>
       <x:c r="I47" s="17" t="str">
-        <x:v>[512,512,512,512]</x:v>
+        <x:v>[4096,4352,4608,4864,5120,5376,5632,5888,6144,6400,6656,6912,7168,7424,7680,7936,8192,8448,8704,8960,9216,9472,9728]</x:v>
       </x:c>
       <x:c r="J47" s="18" t="b">
         <x:v>0</x:v>
@@ -3294,42 +3294,42 @@
       </x:c>
       <x:c r="S47" s="17" t="str"/>
       <x:c r="T47" s="19" t="str">
-        <x:v>SI_WB_046 short2_total_output_plus_one_batch4 覆盖: 短路2临界后一位；进入正常TopK路径 设计: prompt block=4，totalOutput=12，kv block=13，验证刚越过短路边界的行为。</x:v>
+        <x:v>SI_WB_047 batch23_noncausal_varlen_q32_kv8 覆盖: batch=23；non-causal；q/kv多batch变长；较大prompt block；q32/kv8 设计: 用非2次幂batch和递增长度组合，覆盖批量读取、shape最大值推导和non-causal全S2路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="16" t="str">
-        <x:v>SI_WB_047</x:v>
+        <x:v>SI_WB_049</x:v>
       </x:c>
       <x:c r="B48" s="17" t="str">
-        <x:v>batch23_noncausal_varlen_q32_kv8</x:v>
+        <x:v>batch15_decode_prompt_tail_q64_kv4</x:v>
       </x:c>
       <x:c r="C48" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D48" s="17" t="n">
-        <x:v>23</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E48" s="17" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F48" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G48" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304,2432,2560,2688,2816,2944,3072,3200,3328]</x:v>
+        <x:v>[1,1,1,1,1,1,1,1,1,1,1,1,1,1,1]</x:v>
       </x:c>
       <x:c r="H48" s="17" t="str">
-        <x:v>[4096,4352,4608,4864,5120,5376,5632,5888,6144,6400,6656,6912,7168,7424,7680,7936,8192,8448,8704,8960,9216,9472,9728]</x:v>
+        <x:v>[8193,8194,8195,8196,8197,8198,8199,8200,8201,8202,8203,8204,8205,8206,8207]</x:v>
       </x:c>
       <x:c r="I48" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304,2432,2560,2688,2816,2944,3072,3200,3328]</x:v>
+        <x:v>[8193,8194,8195,8196,8197,8198,8199,8200,8201,8202,8203,8204,8205,8206,8207]</x:v>
       </x:c>
       <x:c r="J48" s="18" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K48" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="L48" s="17" t="n">
         <x:v>128</x:v>
@@ -3354,42 +3354,42 @@
       </x:c>
       <x:c r="S48" s="17" t="str"/>
       <x:c r="T48" s="19" t="str">
-        <x:v>SI_WB_047 batch23_noncausal_varlen_q32_kv8 覆盖: batch=23；non-causal；q/kv多batch变长；较大prompt block；q32/kv8 设计: 用非2次幂batch和递增长度组合，覆盖批量读取、shape最大值推导和non-causal全S2路径。</x:v>
+        <x:v>SI_WB_049 batch15_decode_prompt_tail_q64_kv4 覆盖: batch=15；decode；q=1；kv/prompt非128整数倍；q64/kv4 设计: 多batch decode同时覆盖prompt向上取整和不同KV尾块。</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="16" t="str">
-        <x:v>SI_WB_048</x:v>
+        <x:v>SI_WB_050</x:v>
       </x:c>
       <x:c r="B49" s="17" t="str">
-        <x:v>batch21_causal_varlen_q64_kv2</x:v>
+        <x:v>batch4_dynamic_topk_boundary_mix</x:v>
       </x:c>
       <x:c r="C49" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D49" s="17" t="n">
-        <x:v>21</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E49" s="17" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="F49" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G49" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304,2432,2560,2688,2816,2944,3072]</x:v>
+        <x:v>[1024,1024,1024,1024]</x:v>
       </x:c>
       <x:c r="H49" s="17" t="str">
-        <x:v>[8192,8448,8704,8960,9216,9472,9728,9984,10240,10496,10752,11008,11264,11520,11776,12032,12288,12544,12800,13056,13312]</x:v>
+        <x:v>[7040,7168,20352,20480]</x:v>
       </x:c>
       <x:c r="I49" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304,2432,2560,2688,2816,2944,3072]</x:v>
+        <x:v>[7040,7168,20352,20480]</x:v>
       </x:c>
       <x:c r="J49" s="18" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K49" s="17" t="n">
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L49" s="17" t="n">
         <x:v>128</x:v>
@@ -3414,42 +3414,42 @@
       </x:c>
       <x:c r="S49" s="17" t="str"/>
       <x:c r="T49" s="19" t="str">
-        <x:v>SI_WB_048 batch21_causal_varlen_q64_kv2 覆盖: batch=21；causal；q64/kv2大G；S1/S2不等；较大prompt block 设计: 大G场景下同时拉开q/kv长度，验证causal可见S2偏移和GQA映射。</x:v>
+        <x:v>SI_WB_050 batch4_dynamic_topk_boundary_mix 覆盖: 单case混合dynamicTopK边界55/56/159/160；batch=4；q64/kv8 设计: 将small/medium/large分段边界放在同一batch，验证每个batch独立读取prompt长度。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="16" t="str">
-        <x:v>SI_WB_049</x:v>
+        <x:v>SI_WB_051</x:v>
       </x:c>
       <x:c r="B50" s="17" t="str">
-        <x:v>batch15_decode_prompt_tail_q64_kv4</x:v>
+        <x:v>batch24_noncausal_q32_kv2_varlen</x:v>
       </x:c>
       <x:c r="C50" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D50" s="17" t="n">
-        <x:v>15</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E50" s="17" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F50" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G50" s="17" t="str">
-        <x:v>[1,1,1,1,1,1,1,1,1,1,1,1,1,1,1]</x:v>
+        <x:v>[384,448,512,576,640,704,768,832,896,960,1024,1088,1152,1216,1280,1344,1408,1472,1536,1600,1664,1728,1792,1856]</x:v>
       </x:c>
       <x:c r="H50" s="17" t="str">
-        <x:v>[8193,8194,8195,8196,8197,8198,8199,8200,8201,8202,8203,8204,8205,8206,8207]</x:v>
+        <x:v>[2048,2176,2304,2432,2560,2688,2816,2944,3072,3200,3328,3456,3584,3712,3840,3968,4096,4224,4352,4480,4608,4736,4864,4992]</x:v>
       </x:c>
       <x:c r="I50" s="17" t="str">
-        <x:v>[8192,8193,8194,8195,8196,8197,8198,8199,8200,8201,8202,8203,8204,8205,8206]</x:v>
+        <x:v>[2048,2176,2304,2432,2560,2688,2816,2944,3072,3200,3328,3456,3584,3712,3840,3968,4096,4224,4352,4480,4608,4736,4864,4992]</x:v>
       </x:c>
       <x:c r="J50" s="18" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K50" s="17" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L50" s="17" t="n">
         <x:v>128</x:v>
@@ -3474,42 +3474,42 @@
       </x:c>
       <x:c r="S50" s="17" t="str"/>
       <x:c r="T50" s="19" t="str">
-        <x:v>SI_WB_049 batch15_decode_prompt_tail_q64_kv4 覆盖: batch=15；decode；q=1；kv/prompt非128整数倍；q64/kv4 设计: 多batch decode同时覆盖prompt向上取整和不同KV尾块。</x:v>
+        <x:v>SI_WB_051 batch24_noncausal_q32_kv2_varlen 覆盖: batch=24；q32/kv2；non-causal；多batch递增长度 设计: 补齐q32/kv2组合覆盖，验证较大batch下shape最大值推导和完整S2可见范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="16" t="str">
-        <x:v>SI_WB_050</x:v>
+        <x:v>SI_WB_052</x:v>
       </x:c>
       <x:c r="B51" s="17" t="str">
-        <x:v>batch4_dynamic_topk_boundary_mix</x:v>
+        <x:v>batch25_causal_q32_kv2_tail_mix</x:v>
       </x:c>
       <x:c r="C51" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D51" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E51" s="17" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F51" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G51" s="17" t="str">
-        <x:v>[1024,1024,1024,1024]</x:v>
+        <x:v>[129,202,275,348,421,494,567,640,713,786,859,932,1005,1078,1151,1224,1297,1370,1443,1516,1589,1662,1735,1808,1881]</x:v>
       </x:c>
       <x:c r="H51" s="17" t="str">
-        <x:v>[16384,16384,32768,32768]</x:v>
+        <x:v>[1025,1122,1219,1316,1413,1510,1607,1704,1801,1898,1995,2092,2189,2286,2383,2480,2577,2674,2771,2868,2965,3062,3159,3256,3353]</x:v>
       </x:c>
       <x:c r="I51" s="17" t="str">
-        <x:v>[7040,7168,20352,20480]</x:v>
+        <x:v>[1025,1122,1219,1316,1413,1510,1607,1704,1801,1898,1995,2092,2189,2286,2383,2480,2577,2674,2771,2868,2965,3062,3159,3256,3353]</x:v>
       </x:c>
       <x:c r="J51" s="18" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K51" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="L51" s="17" t="n">
         <x:v>128</x:v>
@@ -3534,21 +3534,21 @@
       </x:c>
       <x:c r="S51" s="17" t="str"/>
       <x:c r="T51" s="19" t="str">
-        <x:v>SI_WB_050 batch4_dynamic_topk_boundary_mix 覆盖: 单case混合dynamicTopK边界55/56/159/160；batch=4；q64/kv8 设计: 将small/medium/large分段边界放在同一batch，验证每个batch独立读取prompt长度。</x:v>
+        <x:v>SI_WB_052 batch25_causal_q32_kv2_tail_mix 覆盖: batch=25；q32/kv2；causal；q/kv均非128整数倍 设计: 用非整齐batch和尾块长度组合，验证causal下每个batch独立计算可见S2。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="16" t="str">
-        <x:v>SI_WB_051</x:v>
+        <x:v>SI_WB_053</x:v>
       </x:c>
       <x:c r="B52" s="17" t="str">
-        <x:v>batch24_noncausal_q32_kv2_varlen</x:v>
+        <x:v>batch27_decode_q32_kv2_prompt_tail</x:v>
       </x:c>
       <x:c r="C52" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D52" s="17" t="n">
-        <x:v>24</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E52" s="17" t="n">
         <x:v>32</x:v>
@@ -3557,19 +3557,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G52" s="17" t="str">
-        <x:v>[384,448,512,576,640,704,768,832,896,960,1024,1088,1152,1216,1280,1344,1408,1472,1536,1600,1664,1728,1792,1856]</x:v>
+        <x:v>[1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1]</x:v>
       </x:c>
       <x:c r="H52" s="17" t="str">
-        <x:v>[2048,2176,2304,2432,2560,2688,2816,2944,3072,3200,3328,3456,3584,3712,3840,3968,4096,4224,4352,4480,4608,4736,4864,4992]</x:v>
+        <x:v>[4097,4098,4099,4100,4101,4102,4103,4104,4105,4106,4107,4108,4109,4110,4111,4112,4113,4114,4115,4116,4117,4118,4119,4120,4121,4122,4123]</x:v>
       </x:c>
       <x:c r="I52" s="17" t="str">
-        <x:v>[384,448,512,576,640,704,768,832,896,960,1024,1088,1152,1216,1280,1344,1408,1472,1536,1600,1664,1728,1792,1856]</x:v>
+        <x:v>[4097,4098,4099,4100,4101,4102,4103,4104,4105,4106,4107,4108,4109,4110,4111,4112,4113,4114,4115,4116,4117,4118,4119,4120,4121,4122,4123]</x:v>
       </x:c>
       <x:c r="J52" s="18" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K52" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="L52" s="17" t="n">
         <x:v>128</x:v>
@@ -3594,42 +3594,42 @@
       </x:c>
       <x:c r="S52" s="17" t="str"/>
       <x:c r="T52" s="19" t="str">
-        <x:v>SI_WB_051 batch24_noncausal_q32_kv2_varlen 覆盖: batch=24；q32/kv2；non-causal；多batch递增长度 设计: 补齐q32/kv2组合覆盖，验证较大batch下shape最大值推导和完整S2可见范围。</x:v>
+        <x:v>SI_WB_053 batch27_decode_q32_kv2_prompt_tail 覆盖: batch=27；q32/kv2；decode；prompt和kv均带尾块 设计: 多batch decode下验证num_prompt_tokens按batch读取，并覆盖prompt非128整数倍。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="16" t="str">
-        <x:v>SI_WB_052</x:v>
+        <x:v>SI_WB_054</x:v>
       </x:c>
       <x:c r="B53" s="17" t="str">
-        <x:v>batch25_causal_q32_kv2_tail_mix</x:v>
+        <x:v>batch26_noncausal_q32_kv4_varlen</x:v>
       </x:c>
       <x:c r="C53" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D53" s="17" t="n">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E53" s="17" t="n">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F53" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G53" s="17" t="str">
-        <x:v>[129,202,275,348,421,494,567,640,713,786,859,932,1005,1078,1151,1224,1297,1370,1443,1516,1589,1662,1735,1808,1881]</x:v>
+        <x:v>[512,544,576,608,640,672,704,736,768,800,832,864,896,928,960,992,1024,1056,1088,1120,1152,1184,1216,1248,1280,1312]</x:v>
       </x:c>
       <x:c r="H53" s="17" t="str">
-        <x:v>[1025,1122,1219,1316,1413,1510,1607,1704,1801,1898,1995,2092,2189,2286,2383,2480,2577,2674,2771,2868,2965,3062,3159,3256,3353]</x:v>
+        <x:v>[1536,1632,1728,1824,1920,2016,2112,2208,2304,2400,2496,2592,2688,2784,2880,2976,3072,3168,3264,3360,3456,3552,3648,3744,3840,3936]</x:v>
       </x:c>
       <x:c r="I53" s="17" t="str">
-        <x:v>[129,202,275,348,421,494,567,640,713,786,859,932,1005,1078,1151,1224,1297,1370,1443,1516,1589,1662,1735,1808,1881]</x:v>
+        <x:v>[1536,1632,1728,1824,1920,2016,2112,2208,2304,2400,2496,2592,2688,2784,2880,2976,3072,3168,3264,3360,3456,3552,3648,3744,3840,3936]</x:v>
       </x:c>
       <x:c r="J53" s="18" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K53" s="17" t="n">
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L53" s="17" t="n">
         <x:v>128</x:v>
@@ -3654,36 +3654,36 @@
       </x:c>
       <x:c r="S53" s="17" t="str"/>
       <x:c r="T53" s="19" t="str">
-        <x:v>SI_WB_052 batch25_causal_q32_kv2_tail_mix 覆盖: batch=25；q32/kv2；causal；q/kv均非128整数倍 设计: 用非整齐batch和尾块长度组合，验证causal下每个batch独立计算可见S2。</x:v>
+        <x:v>SI_WB_054 batch26_noncausal_q32_kv4_varlen 覆盖: batch=26；q32/kv4；non-causal；q尾块与kv尾块混合 设计: 补齐q32/kv4组合覆盖，验证中等GQA组下的多batch变长路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="16" t="str">
-        <x:v>SI_WB_053</x:v>
+        <x:v>SI_WB_055</x:v>
       </x:c>
       <x:c r="B54" s="17" t="str">
-        <x:v>batch27_decode_q32_kv2_prompt_tail</x:v>
+        <x:v>batch28_causal_q32_kv4_offset_tail</x:v>
       </x:c>
       <x:c r="C54" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D54" s="17" t="n">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E54" s="17" t="n">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F54" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G54" s="17" t="str">
-        <x:v>[1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1]</x:v>
+        <x:v>[256,313,370,427,484,541,598,655,712,769,826,883,940,997,1054,1111,1168,1225,1282,1339,1396,1453,1510,1567,1624,1681,1738,1795]</x:v>
       </x:c>
       <x:c r="H54" s="17" t="str">
-        <x:v>[4097,4098,4099,4100,4101,4102,4103,4104,4105,4106,4107,4108,4109,4110,4111,4112,4113,4114,4115,4116,4117,4118,4119,4120,4121,4122,4123]</x:v>
+        <x:v>[2048,2139,2230,2321,2412,2503,2594,2685,2776,2867,2958,3049,3140,3231,3322,3413,3504,3595,3686,3777,3868,3959,4050,4141,4232,4323,4414,4505]</x:v>
       </x:c>
       <x:c r="I54" s="17" t="str">
-        <x:v>[4096,4097,4098,4099,4100,4101,4102,4103,4104,4105,4106,4107,4108,4109,4110,4111,4112,4113,4114,4115,4116,4117,4118,4119,4120,4121,4122]</x:v>
+        <x:v>[2048,2139,2230,2321,2412,2503,2594,2685,2776,2867,2958,3049,3140,3231,3322,3413,3504,3595,3686,3777,3868,3959,4050,4141,4232,4323,4414,4505]</x:v>
       </x:c>
       <x:c r="J54" s="18" t="b">
         <x:v>1</x:v>
@@ -3714,21 +3714,21 @@
       </x:c>
       <x:c r="S54" s="17" t="str"/>
       <x:c r="T54" s="19" t="str">
-        <x:v>SI_WB_053 batch27_decode_q32_kv2_prompt_tail 覆盖: batch=27；q32/kv2；decode；prompt和kv均带尾块 设计: 多batch decode下验证num_prompt_tokens按batch读取，并覆盖prompt非128整数倍。</x:v>
+        <x:v>SI_WB_055 batch28_causal_q32_kv4_offset_tail 覆盖: batch=28；q32/kv4；causal；S1/S2不等且均带尾块 设计: 通过非等差块边界长度覆盖causal可见范围偏移和尾块组合。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="16" t="str">
-        <x:v>SI_WB_054</x:v>
+        <x:v>SI_WB_056</x:v>
       </x:c>
       <x:c r="B55" s="17" t="str">
-        <x:v>batch26_noncausal_q32_kv4_varlen</x:v>
+        <x:v>batch30_noncausal_q32_kv4_prompt_tail</x:v>
       </x:c>
       <x:c r="C55" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D55" s="17" t="n">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E55" s="17" t="n">
         <x:v>32</x:v>
@@ -3737,19 +3737,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G55" s="17" t="str">
-        <x:v>[512,544,576,608,640,672,704,736,768,800,832,864,896,928,960,992,1024,1056,1088,1120,1152,1184,1216,1248,1280,1312]</x:v>
+        <x:v>[640,677,714,751,788,825,862,899,936,973,1010,1047,1084,1121,1158,1195,1232,1269,1306,1343,1380,1417,1454,1491,1528,1565,1602,1639,1676,1713]</x:v>
       </x:c>
       <x:c r="H55" s="17" t="str">
-        <x:v>[1536,1632,1728,1824,1920,2016,2112,2208,2304,2400,2496,2592,2688,2784,2880,2976,3072,3168,3264,3360,3456,3552,3648,3744,3840,3936]</x:v>
+        <x:v>[3072,3155,3238,3321,3404,3487,3570,3653,3736,3819,3902,3985,4068,4151,4234,4317,4400,4483,4566,4649,4732,4815,4898,4981,5064,5147,5230,5313,5396,5479]</x:v>
       </x:c>
       <x:c r="I55" s="17" t="str">
-        <x:v>[512,544,576,608,640,672,704,736,768,800,832,864,896,928,960,992,1024,1056,1088,1120,1152,1184,1216,1248,1280,1312]</x:v>
+        <x:v>[3072,3155,3238,3321,3404,3487,3570,3653,3736,3819,3902,3985,4068,4151,4234,4317,4400,4483,4566,4649,4732,4815,4898,4981,5064,5147,5230,5313,5396,5479]</x:v>
       </x:c>
       <x:c r="J55" s="18" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K55" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="L55" s="17" t="n">
         <x:v>128</x:v>
@@ -3774,36 +3774,36 @@
       </x:c>
       <x:c r="S55" s="17" t="str"/>
       <x:c r="T55" s="19" t="str">
-        <x:v>SI_WB_054 batch26_noncausal_q32_kv4_varlen 覆盖: batch=26；q32/kv4；non-causal；q尾块与kv尾块混合 设计: 补齐q32/kv4组合覆盖，验证中等GQA组下的多batch变长路径。</x:v>
+        <x:v>SI_WB_056 batch30_noncausal_q32_kv4_prompt_tail 覆盖: batch=30；q32/kv4；non-causal；prompt不能整除stem_block_size 设计: 大batch下每个batch的prompt长度不同，验证动态TopK预算读取不同prompt block。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="16" t="str">
-        <x:v>SI_WB_055</x:v>
+        <x:v>SI_WB_058</x:v>
       </x:c>
       <x:c r="B56" s="17" t="str">
-        <x:v>batch28_causal_q32_kv4_offset_tail</x:v>
+        <x:v>decode_q64_kv2_1m_tokens</x:v>
       </x:c>
       <x:c r="C56" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D56" s="17" t="n">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E56" s="17" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F56" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G56" s="17" t="str">
-        <x:v>[256,313,370,427,484,541,598,655,712,769,826,883,940,997,1054,1111,1168,1225,1282,1339,1396,1453,1510,1567,1624,1681,1738,1795]</x:v>
+        <x:v>[1]</x:v>
       </x:c>
       <x:c r="H56" s="17" t="str">
-        <x:v>[2048,2139,2230,2321,2412,2503,2594,2685,2776,2867,2958,3049,3140,3231,3322,3413,3504,3595,3686,3777,3868,3959,4050,4141,4232,4323,4414,4505]</x:v>
+        <x:v>[1048576]</x:v>
       </x:c>
       <x:c r="I56" s="17" t="str">
-        <x:v>[256,313,370,427,484,541,598,655,712,769,826,883,940,997,1054,1111,1168,1225,1282,1339,1396,1453,1510,1567,1624,1681,1738,1795]</x:v>
+        <x:v>[1048576]</x:v>
       </x:c>
       <x:c r="J56" s="18" t="b">
         <x:v>1</x:v>
@@ -3834,42 +3834,42 @@
       </x:c>
       <x:c r="S56" s="17" t="str"/>
       <x:c r="T56" s="19" t="str">
-        <x:v>SI_WB_055 batch28_causal_q32_kv4_offset_tail 覆盖: batch=28；q32/kv4；causal；S1/S2不等且均带尾块 设计: 通过非等差块边界长度覆盖causal可见范围偏移和尾块组合。</x:v>
+        <x:v>SI_WB_058 decode_q64_kv2_1m_tokens 覆盖: batch=1；q64/kv2；decode；KV长度达到1M token 设计: 大G decode路径下覆盖1M以内超长KV上限，验证prompt预算长度等于kv长度时的metadata和golden对齐。</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="16" t="str">
-        <x:v>SI_WB_056</x:v>
+        <x:v>SI_WB_059</x:v>
       </x:c>
       <x:c r="B57" s="17" t="str">
-        <x:v>batch30_noncausal_q32_kv4_prompt_tail</x:v>
+        <x:v>batch18_causal_q64_kv2_offset</x:v>
       </x:c>
       <x:c r="C57" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D57" s="17" t="n">
-        <x:v>30</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E57" s="17" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F57" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G57" s="17" t="str">
-        <x:v>[640,677,714,751,788,825,862,899,936,973,1010,1047,1084,1121,1158,1195,1232,1269,1306,1343,1380,1417,1454,1491,1528,1565,1602,1639,1676,1713]</x:v>
+        <x:v>[384,464,544,624,704,784,864,944,1024,1104,1184,1264,1344,1424,1504,1584,1664,1744]</x:v>
       </x:c>
       <x:c r="H57" s="17" t="str">
-        <x:v>[3072,3155,3238,3321,3404,3487,3570,3653,3736,3819,3902,3985,4068,4151,4234,4317,4400,4483,4566,4649,4732,4815,4898,4981,5064,5147,5230,5313,5396,5479]</x:v>
+        <x:v>[8192,8320,8448,8576,8704,8832,8960,9088,9216,9344,9472,9600,9728,9856,9984,10112,10240,10368]</x:v>
       </x:c>
       <x:c r="I57" s="17" t="str">
-        <x:v>[640,677,714,751,788,825,862,899,936,973,1010,1047,1084,1121,1158,1195,1232,1269,1306,1343,1380,1417,1454,1491,1528,1565,1602,1639,1676,1713]</x:v>
+        <x:v>[8192,8320,8448,8576,8704,8832,8960,9088,9216,9344,9472,9600,9728,9856,9984,10112,10240,10368]</x:v>
       </x:c>
       <x:c r="J57" s="18" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K57" s="17" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="L57" s="17" t="n">
         <x:v>128</x:v>
@@ -3894,253 +3894,73 @@
       </x:c>
       <x:c r="S57" s="17" t="str"/>
       <x:c r="T57" s="19" t="str">
-        <x:v>SI_WB_056 batch30_noncausal_q32_kv4_prompt_tail 覆盖: batch=30；q32/kv4；non-causal；prompt不能整除stem_block_size 设计: 大batch下每个batch的prompt长度不同，验证动态TopK预算读取不同prompt block。</x:v>
+        <x:v>SI_WB_059 batch18_causal_q64_kv2_offset 覆盖: batch=18；q64/kv2；causal；S1/S2不等 设计: 最大GQA组下拉开q/kv块数，覆盖因果偏移和TPD衰减路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
-      <x:c r="A58" s="16" t="str">
-        <x:v>SI_WB_057</x:v>
-      </x:c>
-      <x:c r="B58" s="17" t="str">
-        <x:v>batch22_noncausal_q64_kv2_varlen</x:v>
-      </x:c>
-      <x:c r="C58" s="17" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="D58" s="17" t="n">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E58" s="17" t="n">
+      <x:c r="A58" s="20" t="str">
+        <x:v>SI_WB_060</x:v>
+      </x:c>
+      <x:c r="B58" s="21" t="str">
+        <x:v>batch37_noncausal_q64_kv4_small_varlen</x:v>
+      </x:c>
+      <x:c r="C58" s="21" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D58" s="21" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E58" s="21" t="n">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="F58" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G58" s="17" t="str">
-        <x:v>[512,608,704,800,896,992,1088,1184,1280,1376,1472,1568,1664,1760,1856,1952,2048,2144,2240,2336,2432,2528]</x:v>
-      </x:c>
-      <x:c r="H58" s="17" t="str">
-        <x:v>[4096,4256,4416,4576,4736,4896,5056,5216,5376,5536,5696,5856,6016,6176,6336,6496,6656,6816,6976,7136,7296,7456]</x:v>
-      </x:c>
-      <x:c r="I58" s="17" t="str">
-        <x:v>[512,608,704,800,896,992,1088,1184,1280,1376,1472,1568,1664,1760,1856,1952,2048,2144,2240,2336,2432,2528]</x:v>
-      </x:c>
-      <x:c r="J58" s="18" t="b">
+      <x:c r="F58" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G58" s="21" t="str">
+        <x:v>[128,136,144,152,160,168,176,184,192,200,208,216,224,232,240,248,256,264,272,280,288,296,304,312,320,328,336,344,352,360,368,376,384,392,400,408,416]</x:v>
+      </x:c>
+      <x:c r="H58" s="21" t="str">
+        <x:v>[512,520,528,536,544,552,560,568,576,584,592,600,608,616,624,632,640,648,656,664,672,680,688,696,704,712,720,728,736,744,752,760,768,776,784,792,800]</x:v>
+      </x:c>
+      <x:c r="I58" s="21" t="str">
+        <x:v>[512,520,528,536,544,552,560,568,576,584,592,600,608,616,624,632,640,648,656,664,672,680,688,696,704,712,720,728,736,744,752,760,768,776,784,792,800]</x:v>
+      </x:c>
+      <x:c r="J58" s="22" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K58" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L58" s="17" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="M58" s="17" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="N58" s="17" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="O58" s="17" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P58" s="17" t="str">
-        <x:v>BF16</x:v>
-      </x:c>
-      <x:c r="Q58" s="17" t="str">
-        <x:v>BF16</x:v>
-      </x:c>
-      <x:c r="R58" s="17" t="str">
-        <x:v>FP32</x:v>
-      </x:c>
-      <x:c r="S58" s="17" t="str"/>
-      <x:c r="T58" s="19" t="str">
-        <x:v>SI_WB_057 batch22_noncausal_q64_kv2_varlen 覆盖: batch=22；q64/kv2；non-causal；最大GQA组 设计: 补齐q64/kv2组合覆盖，验证大G场景下多batch变长和完整S2路径。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="15" hidden="0" customHeight="1">
-      <x:c r="A59" s="16" t="str">
-        <x:v>SI_WB_058</x:v>
-      </x:c>
-      <x:c r="B59" s="17" t="str">
-        <x:v>decode_q64_kv2_16k_blocks</x:v>
-      </x:c>
-      <x:c r="C59" s="17" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="D59" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E59" s="17" t="n">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="F59" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G59" s="17" t="str">
-        <x:v>[1]</x:v>
-      </x:c>
-      <x:c r="H59" s="17" t="str">
-        <x:v>[2097152]</x:v>
-      </x:c>
-      <x:c r="I59" s="17" t="str">
-        <x:v>[2097151]</x:v>
-      </x:c>
-      <x:c r="J59" s="18" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K59" s="17" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="L59" s="17" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="M59" s="17" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="N59" s="17" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="O59" s="17" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P59" s="17" t="str">
-        <x:v>BF16</x:v>
-      </x:c>
-      <x:c r="Q59" s="17" t="str">
-        <x:v>BF16</x:v>
-      </x:c>
-      <x:c r="R59" s="17" t="str">
-        <x:v>FP32</x:v>
-      </x:c>
-      <x:c r="S59" s="17" t="str"/>
-      <x:c r="T59" s="19" t="str">
-        <x:v>SI_WB_058 decode_q64_kv2_16k_blocks 覆盖: batch=1；q64/kv2；decode；KV长度达到16384个block 设计: 大G decode路径下覆盖超长KV，验证prompt长度与kv长度错开一位时的metadata和golden对齐。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="15" hidden="0" customHeight="1">
-      <x:c r="A60" s="16" t="str">
-        <x:v>SI_WB_059</x:v>
-      </x:c>
-      <x:c r="B60" s="17" t="str">
-        <x:v>batch18_causal_q64_kv2_offset</x:v>
-      </x:c>
-      <x:c r="C60" s="17" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="D60" s="17" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E60" s="17" t="n">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="F60" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G60" s="17" t="str">
-        <x:v>[384,464,544,624,704,784,864,944,1024,1104,1184,1264,1344,1424,1504,1584,1664,1744]</x:v>
-      </x:c>
-      <x:c r="H60" s="17" t="str">
-        <x:v>[8192,8320,8448,8576,8704,8832,8960,9088,9216,9344,9472,9600,9728,9856,9984,10112,10240,10368]</x:v>
-      </x:c>
-      <x:c r="I60" s="17" t="str">
-        <x:v>[384,464,544,624,704,784,864,944,1024,1104,1184,1264,1344,1424,1504,1584,1664,1744]</x:v>
-      </x:c>
-      <x:c r="J60" s="18" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K60" s="17" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="L60" s="17" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="M60" s="17" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="N60" s="17" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="O60" s="17" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P60" s="17" t="str">
-        <x:v>BF16</x:v>
-      </x:c>
-      <x:c r="Q60" s="17" t="str">
-        <x:v>BF16</x:v>
-      </x:c>
-      <x:c r="R60" s="17" t="str">
-        <x:v>FP32</x:v>
-      </x:c>
-      <x:c r="S60" s="17" t="str"/>
-      <x:c r="T60" s="19" t="str">
-        <x:v>SI_WB_059 batch18_causal_q64_kv2_offset 覆盖: batch=18；q64/kv2；causal；S1/S2不等 设计: 最大GQA组下拉开q/kv块数，覆盖因果偏移和TPD衰减路径。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="15" hidden="0" customHeight="1">
-      <x:c r="A61" s="20" t="str">
-        <x:v>SI_WB_060</x:v>
-      </x:c>
-      <x:c r="B61" s="21" t="str">
-        <x:v>batch37_noncausal_q64_kv4_small_varlen</x:v>
-      </x:c>
-      <x:c r="C61" s="21" t="str">
-        <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="D61" s="21" t="n">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="E61" s="21" t="n">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="F61" s="21" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G61" s="21" t="str">
-        <x:v>[128,136,144,152,160,168,176,184,192,200,208,216,224,232,240,248,256,264,272,280,288,296,304,312,320,328,336,344,352,360,368,376,384,392,400,408,416]</x:v>
-      </x:c>
-      <x:c r="H61" s="21" t="str">
-        <x:v>[512,520,528,536,544,552,560,568,576,584,592,600,608,616,624,632,640,648,656,664,672,680,688,696,704,712,720,728,736,744,752,760,768,776,784,792,800]</x:v>
-      </x:c>
-      <x:c r="I61" s="21" t="str">
-        <x:v>[128,136,144,152,160,168,176,184,192,200,208,216,224,232,240,248,256,264,272,280,288,296,304,312,320,328,336,344,352,360,368,376,384,392,400,408,416]</x:v>
-      </x:c>
-      <x:c r="J61" s="22" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K61" s="21" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L61" s="21" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="M61" s="21" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="N61" s="21" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="O61" s="21" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P61" s="21" t="str">
-        <x:v>BF16</x:v>
-      </x:c>
-      <x:c r="Q61" s="21" t="str">
-        <x:v>BF16</x:v>
-      </x:c>
-      <x:c r="R61" s="21" t="str">
-        <x:v>FP32</x:v>
-      </x:c>
-      <x:c r="S61" s="21" t="str"/>
-      <x:c r="T61" s="23" t="str">
+      <x:c r="K58" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L58" s="21" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="M58" s="21" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N58" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O58" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P58" s="21" t="str">
+        <x:v>BF16</x:v>
+      </x:c>
+      <x:c r="Q58" s="21" t="str">
+        <x:v>BF16</x:v>
+      </x:c>
+      <x:c r="R58" s="21" t="str">
+        <x:v>FP32</x:v>
+      </x:c>
+      <x:c r="S58" s="21" t="str"/>
+      <x:c r="T58" s="23" t="str">
         <x:v>SI_WB_060 batch37_noncausal_q64_kv4_small_varlen 覆盖: batch=37；q64/kv4；短序列多batch；非2次幂batch 设计: 用较小序列控制运行成本，同时覆盖高batch数量和q64/kv4组合。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5de71e7fd3543cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R534c94d593944078"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine StemIndexer pytest sequence coverage
</commit_message>
<xml_diff>
--- a/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
+++ b/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R9c1718c6bb544f4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re6b79c4f76304a16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -613,13 +613,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G3" s="17" t="str">
-        <x:v>[1153]</x:v>
+        <x:v>[147585]</x:v>
       </x:c>
       <x:c r="H3" s="17" t="str">
-        <x:v>[2048]</x:v>
+        <x:v>[262144]</x:v>
       </x:c>
       <x:c r="I3" s="17" t="str">
-        <x:v>[2048]</x:v>
+        <x:v>[262144]</x:v>
       </x:c>
       <x:c r="J3" s="18" t="b">
         <x:v>1</x:v>
@@ -673,13 +673,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G4" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[131072]</x:v>
       </x:c>
       <x:c r="H4" s="17" t="str">
-        <x:v>[2305]</x:v>
+        <x:v>[295041]</x:v>
       </x:c>
       <x:c r="I4" s="17" t="str">
-        <x:v>[2305]</x:v>
+        <x:v>[295041]</x:v>
       </x:c>
       <x:c r="J4" s="18" t="b">
         <x:v>1</x:v>
@@ -733,13 +733,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G5" s="17" t="str">
-        <x:v>[129,257,385,513,641,769,897]</x:v>
+        <x:v>[16513, 32897, 49281, 65665, 82049, 98433, 114817]</x:v>
       </x:c>
       <x:c r="H5" s="17" t="str">
-        <x:v>[257,513,769,1025,1281,1537,1793]</x:v>
+        <x:v>[32897, 65665, 98433, 131201, 163969, 196737, 229505]</x:v>
       </x:c>
       <x:c r="I5" s="17" t="str">
-        <x:v>[257,513,769,1025,1281,1537,1793]</x:v>
+        <x:v>[32897, 65665, 98433, 131201, 163969, 196737, 229505]</x:v>
       </x:c>
       <x:c r="J5" s="18" t="b">
         <x:v>1</x:v>
@@ -770,7 +770,7 @@
       </x:c>
       <x:c r="S5" s="17" t="str"/>
       <x:c r="T5" s="19" t="str">
-        <x:v>SI_WB_004 q_and_kv_tail_batch7_varlen 覆盖: q尾块；kv尾块；短序列；forced集合可能重叠 设计: q 和 kv 同时存在尾块，且块数较少，可同时覆盖尾块和短序列 forced 去重。</x:v>
+        <x:v>SI_WB_004 q_and_kv_tail_batch7_varlen 覆盖: q尾块；kv尾块；batch=7变长；长KV下causal偏移 设计: q 和 kv 同时存在尾块，并将KV/prompt拉到长序列量级，验证多batch变长尾块路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -793,13 +793,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G6" s="17" t="str">
-        <x:v>[512,512,512,512,512,512,512,512]</x:v>
+        <x:v>[512, 512, 512, 512, 512, 512, 512, 512]</x:v>
       </x:c>
       <x:c r="H6" s="17" t="str">
-        <x:v>[512,512,512,512,512,512,512,512]</x:v>
+        <x:v>[512, 512, 512, 512, 512, 512, 512, 512]</x:v>
       </x:c>
       <x:c r="I6" s="17" t="str">
-        <x:v>[512,512,512,512,512,512,512,512]</x:v>
+        <x:v>[512, 512, 512, 512, 512, 512, 512, 512]</x:v>
       </x:c>
       <x:c r="J6" s="18" t="b">
         <x:v>0</x:v>
@@ -853,13 +853,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G7" s="17" t="str">
-        <x:v>[640,768,896,1024,1152]</x:v>
+        <x:v>[640, 768, 896, 1024, 1152]</x:v>
       </x:c>
       <x:c r="H7" s="17" t="str">
-        <x:v>[896,1024,1152,1280,1408]</x:v>
+        <x:v>[896, 1024, 1152, 1280, 1408]</x:v>
       </x:c>
       <x:c r="I7" s="17" t="str">
-        <x:v>[896,1024,1152,1280,1408]</x:v>
+        <x:v>[896, 1024, 1152, 1280, 1408]</x:v>
       </x:c>
       <x:c r="J7" s="18" t="b">
         <x:v>0</x:v>
@@ -913,13 +913,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G8" s="17" t="str">
-        <x:v>[512,640,769,896,1025,1153,1281,1409,1537,1665,1793]</x:v>
+        <x:v>[512, 640, 769, 896, 1025, 1153, 1281, 1409, 1537, 1665, 1793]</x:v>
       </x:c>
       <x:c r="H8" s="17" t="str">
-        <x:v>[2048,2305,2561,2817,3073,3329,3585,3841,4097,4353,4609]</x:v>
+        <x:v>[2048, 2305, 2561, 2817, 3073, 3329, 3585, 3841, 4097, 4353, 4609]</x:v>
       </x:c>
       <x:c r="I8" s="17" t="str">
-        <x:v>[2048,2305,2561,2817,3073,3329,3585,3841,4097,4353,4609]</x:v>
+        <x:v>[2048, 2305, 2561, 2817, 3073, 3329, 3585, 3841, 4097, 4353, 4609]</x:v>
       </x:c>
       <x:c r="J8" s="18" t="b">
         <x:v>0</x:v>
@@ -973,13 +973,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G9" s="17" t="str">
-        <x:v>[128,129,130,160,192,224,225,240,248,256]</x:v>
+        <x:v>[128, 129, 130, 160, 192, 224, 225, 240, 248, 256]</x:v>
       </x:c>
       <x:c r="H9" s="17" t="str">
-        <x:v>[256,256,256,256,256,256,256,256,256,256]</x:v>
+        <x:v>[256, 256, 256, 256, 256, 256, 256, 256, 256, 256]</x:v>
       </x:c>
       <x:c r="I9" s="17" t="str">
-        <x:v>[256,256,256,256,256,256,256,256,256,256]</x:v>
+        <x:v>[256, 256, 256, 256, 256, 256, 256, 256, 256, 256]</x:v>
       </x:c>
       <x:c r="J9" s="18" t="b">
         <x:v>0</x:v>
@@ -1033,13 +1033,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G10" s="17" t="str">
-        <x:v>[1024]</x:v>
+        <x:v>[131072]</x:v>
       </x:c>
       <x:c r="H10" s="17" t="str">
-        <x:v>[4096]</x:v>
+        <x:v>[524288]</x:v>
       </x:c>
       <x:c r="I10" s="17" t="str">
-        <x:v>[4096]</x:v>
+        <x:v>[524288]</x:v>
       </x:c>
       <x:c r="J10" s="18" t="b">
         <x:v>1</x:v>
@@ -1093,13 +1093,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="17" t="str">
-        <x:v>[1024,1152,1280,1408,1536,1664]</x:v>
+        <x:v>[1024, 1152, 1280, 1408, 1536, 1664]</x:v>
       </x:c>
       <x:c r="H11" s="17" t="str">
-        <x:v>[4096,4353,4609,4865,5121,5377]</x:v>
+        <x:v>[524288, 557185, 589953, 622721, 655489, 688257]</x:v>
       </x:c>
       <x:c r="I11" s="17" t="str">
-        <x:v>[4096,4353,4609,4865,5121,5377]</x:v>
+        <x:v>[524288, 557185, 589953, 622721, 655489, 688257]</x:v>
       </x:c>
       <x:c r="J11" s="18" t="b">
         <x:v>0</x:v>
@@ -1130,7 +1130,7 @@
       </x:c>
       <x:c r="S11" s="17" t="str"/>
       <x:c r="T11" s="19" t="str">
-        <x:v>SI_WB_010 noncausal_full_kv_window_batch6_g16 覆盖: causal=false；每个q块可见完整kv；window落在全局kv尾部 设计: 和 causal=true 同 shape 对照，验证非因果路径使用完整 kv 范围。</x:v>
+        <x:v>SI_WB_010 noncausal_full_kv_window_batch6_g16 覆盖: causal=false；每个q块可见完整kv；window落在全局kv尾部 设计: 保持q长度较小并拉长KV/prompt，验证非因果路径使用完整长KV范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1333,13 +1333,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G15" s="17" t="str">
-        <x:v>[512,1024]</x:v>
+        <x:v>[512, 1024]</x:v>
       </x:c>
       <x:c r="H15" s="17" t="str">
-        <x:v>[16384,16384]</x:v>
+        <x:v>[16384, 16384]</x:v>
       </x:c>
       <x:c r="I15" s="17" t="str">
-        <x:v>[16384,16384]</x:v>
+        <x:v>[16384, 16384]</x:v>
       </x:c>
       <x:c r="J15" s="18" t="b">
         <x:v>1</x:v>
@@ -1393,13 +1393,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G16" s="17" t="str">
-        <x:v>[512,1024]</x:v>
+        <x:v>[512, 1024]</x:v>
       </x:c>
       <x:c r="H16" s="17" t="str">
-        <x:v>[16385,16385]</x:v>
+        <x:v>[16385, 16385]</x:v>
       </x:c>
       <x:c r="I16" s="17" t="str">
-        <x:v>[16385,16385]</x:v>
+        <x:v>[16385, 16385]</x:v>
       </x:c>
       <x:c r="J16" s="18" t="b">
         <x:v>1</x:v>
@@ -1453,13 +1453,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>[512,1024]</x:v>
+        <x:v>[512, 1024]</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
-        <x:v>[32768,32768]</x:v>
+        <x:v>[32768, 32768]</x:v>
       </x:c>
       <x:c r="I17" s="17" t="str">
-        <x:v>[32768,32768]</x:v>
+        <x:v>[32768, 32768]</x:v>
       </x:c>
       <x:c r="J17" s="18" t="b">
         <x:v>1</x:v>
@@ -1513,13 +1513,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G18" s="17" t="str">
-        <x:v>[512,1024]</x:v>
+        <x:v>[512, 1024]</x:v>
       </x:c>
       <x:c r="H18" s="17" t="str">
-        <x:v>[32769,32769]</x:v>
+        <x:v>[32769, 32769]</x:v>
       </x:c>
       <x:c r="I18" s="17" t="str">
-        <x:v>[32769,32769]</x:v>
+        <x:v>[32769, 32769]</x:v>
       </x:c>
       <x:c r="J18" s="18" t="b">
         <x:v>1</x:v>
@@ -1813,13 +1813,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G23" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048]</x:v>
+        <x:v>[512, 640, 768, 896, 1024, 1152, 1280, 1408, 1536, 1664, 1792, 1920, 2048]</x:v>
       </x:c>
       <x:c r="H23" s="17" t="str">
-        <x:v>[2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608,4864,5120]</x:v>
+        <x:v>[262144, 294912, 327680, 360448, 393216, 425984, 458752, 491520, 524288, 557056, 589824, 622592, 655360]</x:v>
       </x:c>
       <x:c r="I23" s="17" t="str">
-        <x:v>[2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608,4864,5120]</x:v>
+        <x:v>[262144, 294912, 327680, 360448, 393216, 425984, 458752, 491520, 524288, 557056, 589824, 622592, 655360]</x:v>
       </x:c>
       <x:c r="J23" s="18" t="b">
         <x:v>1</x:v>
@@ -1873,13 +1873,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G24" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176]</x:v>
+        <x:v>[512, 640, 768, 896, 1024, 1152, 1280, 1408, 1536, 1664, 1792, 1920, 2048, 2176]</x:v>
       </x:c>
       <x:c r="H24" s="17" t="str">
-        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352]</x:v>
+        <x:v>[131072, 163840, 196608, 229376, 262144, 294912, 327680, 360448, 393216, 425984, 458752, 491520, 524288, 557056]</x:v>
       </x:c>
       <x:c r="I24" s="17" t="str">
-        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352]</x:v>
+        <x:v>[131072, 163840, 196608, 229376, 262144, 294912, 327680, 360448, 393216, 425984, 458752, 491520, 524288, 557056]</x:v>
       </x:c>
       <x:c r="J24" s="18" t="b">
         <x:v>1</x:v>
@@ -1933,13 +1933,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G25" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536]</x:v>
+        <x:v>[512, 640, 768, 896, 1024, 1152, 1280, 1408, 1536]</x:v>
       </x:c>
       <x:c r="H25" s="17" t="str">
-        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072]</x:v>
+        <x:v>[131072, 163840, 196608, 229376, 262144, 294912, 327680, 360448, 393216]</x:v>
       </x:c>
       <x:c r="I25" s="17" t="str">
-        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072]</x:v>
+        <x:v>[131072, 163840, 196608, 229376, 262144, 294912, 327680, 360448, 393216]</x:v>
       </x:c>
       <x:c r="J25" s="18" t="b">
         <x:v>1</x:v>
@@ -1993,13 +1993,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G26" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304]</x:v>
+        <x:v>[512, 640, 768, 896, 1024, 1152, 1280, 1408, 1536, 1664, 1792, 1920, 2048, 2176, 2304]</x:v>
       </x:c>
       <x:c r="H26" s="17" t="str">
-        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608]</x:v>
+        <x:v>[131072, 163840, 196608, 229376, 262144, 294912, 327680, 360448, 393216, 425984, 458752, 491520, 524288, 557056, 589824]</x:v>
       </x:c>
       <x:c r="I26" s="17" t="str">
-        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608]</x:v>
+        <x:v>[131072, 163840, 196608, 229376, 262144, 294912, 327680, 360448, 393216, 425984, 458752, 491520, 524288, 557056, 589824]</x:v>
       </x:c>
       <x:c r="J26" s="18" t="b">
         <x:v>1</x:v>
@@ -2053,13 +2053,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G27" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304,2432]</x:v>
+        <x:v>[512, 640, 768, 896, 1024, 1152, 1280, 1408, 1536, 1664, 1792, 1920, 2048, 2176, 2304, 2432]</x:v>
       </x:c>
       <x:c r="H27" s="17" t="str">
-        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608,4864]</x:v>
+        <x:v>[131072, 163840, 196608, 229376, 262144, 294912, 327680, 360448, 393216, 425984, 458752, 491520, 524288, 557056, 589824, 622592]</x:v>
       </x:c>
       <x:c r="I27" s="17" t="str">
-        <x:v>[1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608,4864]</x:v>
+        <x:v>[131072, 163840, 196608, 229376, 262144, 294912, 327680, 360448, 393216, 425984, 458752, 491520, 524288, 557056, 589824, 622592]</x:v>
       </x:c>
       <x:c r="J27" s="18" t="b">
         <x:v>1</x:v>
@@ -2113,13 +2113,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G28" s="17" t="str">
-        <x:v>[256,384,512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304]</x:v>
+        <x:v>[256, 384, 512, 640, 768, 896, 1024, 1152, 1280, 1408, 1536, 1664, 1792, 1920, 2048, 2176, 2304]</x:v>
       </x:c>
       <x:c r="H28" s="17" t="str">
-        <x:v>[512,768,1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608]</x:v>
+        <x:v>[65536, 98304, 131072, 163840, 196608, 229376, 262144, 294912, 327680, 360448, 393216, 425984, 458752, 491520, 524288, 557056, 589824]</x:v>
       </x:c>
       <x:c r="I28" s="17" t="str">
-        <x:v>[512,768,1024,1280,1536,1792,2048,2304,2560,2816,3072,3328,3584,3840,4096,4352,4608]</x:v>
+        <x:v>[65536, 98304, 131072, 163840, 196608, 229376, 262144, 294912, 327680, 360448, 393216, 425984, 458752, 491520, 524288, 557056, 589824]</x:v>
       </x:c>
       <x:c r="J28" s="18" t="b">
         <x:v>1</x:v>
@@ -2173,13 +2173,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G29" s="17" t="str">
-        <x:v>[512,1,640,1,768,1,896,1,1024,1,1152,1,1280,1,1408,1,1536,1,1664]</x:v>
+        <x:v>[512, 1, 640, 1, 768, 1, 896, 1, 1024, 1, 1152, 1, 1280, 1, 1408, 1, 1536, 1, 1664]</x:v>
       </x:c>
       <x:c r="H29" s="17" t="str">
-        <x:v>[1024,8193,1280,8194,1536,8195,1792,8196,2048,8197,2304,8198,2560,8199,2816,8200,3072,8201,3328]</x:v>
+        <x:v>[1024, 8193, 1280, 8194, 1536, 8195, 1792, 8196, 2048, 8197, 2304, 8198, 2560, 8199, 2816, 8200, 3072, 8201, 3328]</x:v>
       </x:c>
       <x:c r="I29" s="17" t="str">
-        <x:v>[1024,8193,1280,8194,1536,8195,1792,8196,2048,8197,2304,8198,2560,8199,2816,8200,3072,8201,3328]</x:v>
+        <x:v>[1024, 8193, 1280, 8194, 1536, 8195, 1792, 8196, 2048, 8197, 2304, 8198, 2560, 8199, 2816, 8200, 3072, 8201, 3328]</x:v>
       </x:c>
       <x:c r="J29" s="18" t="b">
         <x:v>1</x:v>
@@ -2837,13 +2837,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G40" s="17" t="str">
-        <x:v>[128,513,1,640,1,768,1,896,1,1024,1,1152]</x:v>
+        <x:v>[128, 513, 1, 640, 1, 768, 1, 896, 1, 1024, 1, 1152]</x:v>
       </x:c>
       <x:c r="H40" s="17" t="str">
-        <x:v>[512,1025,8194,1280,8195,1536,8196,1792,8197,2048,8198,2304]</x:v>
+        <x:v>[512, 1025, 8194, 1280, 8195, 1536, 8196, 1792, 8197, 2048, 8198, 2304]</x:v>
       </x:c>
       <x:c r="I40" s="17" t="str">
-        <x:v>[512,1025,8194,1280,8195,1536,8196,1792,8197,2048,8198,2304]</x:v>
+        <x:v>[512, 1025, 8194, 1280, 8195, 1536, 8196, 1792, 8197, 2048, 8198, 2304]</x:v>
       </x:c>
       <x:c r="J40" s="18" t="b">
         <x:v>1</x:v>
@@ -2897,13 +2897,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G41" s="17" t="str">
-        <x:v>[768,1153,1537]</x:v>
+        <x:v>[768, 1153, 1537]</x:v>
       </x:c>
       <x:c r="H41" s="17" t="str">
-        <x:v>[1793,2305,2817]</x:v>
+        <x:v>[1793, 2305, 2817]</x:v>
       </x:c>
       <x:c r="I41" s="17" t="str">
-        <x:v>[1793,2305,2817]</x:v>
+        <x:v>[1793, 2305, 2817]</x:v>
       </x:c>
       <x:c r="J41" s="18" t="b">
         <x:v>1</x:v>
@@ -2957,13 +2957,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G42" s="17" t="str">
-        <x:v>[641,769,897,1025,1153]</x:v>
+        <x:v>[641, 769, 897, 1025, 1153]</x:v>
       </x:c>
       <x:c r="H42" s="17" t="str">
-        <x:v>[1537,1793,2049,2305,2561]</x:v>
+        <x:v>[1537, 1793, 2049, 2305, 2561]</x:v>
       </x:c>
       <x:c r="I42" s="17" t="str">
-        <x:v>[1537,1793,2049,2305,2561]</x:v>
+        <x:v>[1537, 1793, 2049, 2305, 2561]</x:v>
       </x:c>
       <x:c r="J42" s="18" t="b">
         <x:v>1</x:v>
@@ -3137,13 +3137,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G45" s="17" t="str">
-        <x:v>[512,512,512,512]</x:v>
+        <x:v>[512, 512, 512, 512]</x:v>
       </x:c>
       <x:c r="H45" s="17" t="str">
-        <x:v>[8320,8320,8320,8320]</x:v>
+        <x:v>[8320, 8320, 8320, 8320]</x:v>
       </x:c>
       <x:c r="I45" s="17" t="str">
-        <x:v>[17280,17280,17280,17280]</x:v>
+        <x:v>[17280, 17280, 17280, 17280]</x:v>
       </x:c>
       <x:c r="J45" s="18" t="b">
         <x:v>0</x:v>
@@ -3197,13 +3197,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G46" s="17" t="str">
-        <x:v>[512,512,512,512]</x:v>
+        <x:v>[512, 512, 512, 512]</x:v>
       </x:c>
       <x:c r="H46" s="17" t="str">
-        <x:v>[8448,8448,8448,8448]</x:v>
+        <x:v>[8448, 8448, 8448, 8448]</x:v>
       </x:c>
       <x:c r="I46" s="17" t="str">
-        <x:v>[17280,17280,17280,17280]</x:v>
+        <x:v>[17280, 17280, 17280, 17280]</x:v>
       </x:c>
       <x:c r="J46" s="18" t="b">
         <x:v>0</x:v>
@@ -3257,13 +3257,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G47" s="17" t="str">
-        <x:v>[512,640,768,896,1024,1152,1280,1408,1536,1664,1792,1920,2048,2176,2304,2432,2560,2688,2816,2944,3072,3200,3328]</x:v>
+        <x:v>[512, 640, 768, 896, 1024, 1152, 1280, 1408, 1536, 1664, 1792, 1920, 2048, 2176, 2304, 2432, 2560, 2688, 2816, 2944, 3072, 3200, 3328]</x:v>
       </x:c>
       <x:c r="H47" s="17" t="str">
-        <x:v>[4096,4352,4608,4864,5120,5376,5632,5888,6144,6400,6656,6912,7168,7424,7680,7936,8192,8448,8704,8960,9216,9472,9728]</x:v>
+        <x:v>[4096, 4352, 4608, 4864, 5120, 5376, 5632, 5888, 6144, 6400, 6656, 6912, 7168, 7424, 7680, 7936, 8192, 8448, 8704, 8960, 9216, 9472, 9728]</x:v>
       </x:c>
       <x:c r="I47" s="17" t="str">
-        <x:v>[4096,4352,4608,4864,5120,5376,5632,5888,6144,6400,6656,6912,7168,7424,7680,7936,8192,8448,8704,8960,9216,9472,9728]</x:v>
+        <x:v>[4096, 4352, 4608, 4864, 5120, 5376, 5632, 5888, 6144, 6400, 6656, 6912, 7168, 7424, 7680, 7936, 8192, 8448, 8704, 8960, 9216, 9472, 9728]</x:v>
       </x:c>
       <x:c r="J47" s="18" t="b">
         <x:v>0</x:v>
@@ -3317,13 +3317,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G48" s="17" t="str">
-        <x:v>[1,1,1,1,1,1,1,1,1,1,1,1,1,1,1]</x:v>
+        <x:v>[1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1]</x:v>
       </x:c>
       <x:c r="H48" s="17" t="str">
-        <x:v>[8193,8194,8195,8196,8197,8198,8199,8200,8201,8202,8203,8204,8205,8206,8207]</x:v>
+        <x:v>[8193, 8194, 8195, 8196, 8197, 8198, 8199, 8200, 8201, 8202, 8203, 8204, 8205, 8206, 8207]</x:v>
       </x:c>
       <x:c r="I48" s="17" t="str">
-        <x:v>[8193,8194,8195,8196,8197,8198,8199,8200,8201,8202,8203,8204,8205,8206,8207]</x:v>
+        <x:v>[8193, 8194, 8195, 8196, 8197, 8198, 8199, 8200, 8201, 8202, 8203, 8204, 8205, 8206, 8207]</x:v>
       </x:c>
       <x:c r="J48" s="18" t="b">
         <x:v>1</x:v>
@@ -3377,13 +3377,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G49" s="17" t="str">
-        <x:v>[1024,1024,1024,1024]</x:v>
+        <x:v>[1024, 1024, 1024, 1024]</x:v>
       </x:c>
       <x:c r="H49" s="17" t="str">
-        <x:v>[7040,7168,20352,20480]</x:v>
+        <x:v>[7040, 7168, 20352, 20480]</x:v>
       </x:c>
       <x:c r="I49" s="17" t="str">
-        <x:v>[7040,7168,20352,20480]</x:v>
+        <x:v>[7040, 7168, 20352, 20480]</x:v>
       </x:c>
       <x:c r="J49" s="18" t="b">
         <x:v>0</x:v>
@@ -3437,13 +3437,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G50" s="17" t="str">
-        <x:v>[384,448,512,576,640,704,768,832,896,960,1024,1088,1152,1216,1280,1344,1408,1472,1536,1600,1664,1728,1792,1856]</x:v>
+        <x:v>[384, 448, 512, 576, 640, 704, 768, 832, 896, 960, 1024, 1088, 1152, 1216, 1280, 1344, 1408, 1472, 1536, 1600, 1664, 1728, 1792, 1856]</x:v>
       </x:c>
       <x:c r="H50" s="17" t="str">
-        <x:v>[2048,2176,2304,2432,2560,2688,2816,2944,3072,3200,3328,3456,3584,3712,3840,3968,4096,4224,4352,4480,4608,4736,4864,4992]</x:v>
+        <x:v>[262144, 278528, 294912, 311296, 327680, 344064, 360448, 376832, 393216, 409600, 425984, 442368, 458752, 475136, 491520, 507904, 524288, 540672, 557056, 573440, 589824, 606208, 622592, 638976]</x:v>
       </x:c>
       <x:c r="I50" s="17" t="str">
-        <x:v>[2048,2176,2304,2432,2560,2688,2816,2944,3072,3200,3328,3456,3584,3712,3840,3968,4096,4224,4352,4480,4608,4736,4864,4992]</x:v>
+        <x:v>[262144, 278528, 294912, 311296, 327680, 344064, 360448, 376832, 393216, 409600, 425984, 442368, 458752, 475136, 491520, 507904, 524288, 540672, 557056, 573440, 589824, 606208, 622592, 638976]</x:v>
       </x:c>
       <x:c r="J50" s="18" t="b">
         <x:v>0</x:v>
@@ -3497,13 +3497,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G51" s="17" t="str">
-        <x:v>[129,202,275,348,421,494,567,640,713,786,859,932,1005,1078,1151,1224,1297,1370,1443,1516,1589,1662,1735,1808,1881]</x:v>
+        <x:v>[129, 202, 275, 348, 421, 494, 567, 640, 713, 786, 859, 932, 1005, 1078, 1151, 1224, 1297, 1370, 1443, 1516, 1589, 1662, 1735, 1808, 1881]</x:v>
       </x:c>
       <x:c r="H51" s="17" t="str">
-        <x:v>[1025,1122,1219,1316,1413,1510,1607,1704,1801,1898,1995,2092,2189,2286,2383,2480,2577,2674,2771,2868,2965,3062,3159,3256,3353]</x:v>
+        <x:v>[131201, 143714, 156099, 168484, 180869, 193382, 205767, 218152, 230537, 243050, 255435, 267820, 280205, 292718, 305103, 317488, 329873, 342386, 354771, 367156, 379541, 392054, 404439, 416824, 429209]</x:v>
       </x:c>
       <x:c r="I51" s="17" t="str">
-        <x:v>[1025,1122,1219,1316,1413,1510,1607,1704,1801,1898,1995,2092,2189,2286,2383,2480,2577,2674,2771,2868,2965,3062,3159,3256,3353]</x:v>
+        <x:v>[131201, 143714, 156099, 168484, 180869, 193382, 205767, 218152, 230537, 243050, 255435, 267820, 280205, 292718, 305103, 317488, 329873, 342386, 354771, 367156, 379541, 392054, 404439, 416824, 429209]</x:v>
       </x:c>
       <x:c r="J51" s="18" t="b">
         <x:v>1</x:v>
@@ -3557,13 +3557,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G52" s="17" t="str">
-        <x:v>[1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1]</x:v>
+        <x:v>[1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1]</x:v>
       </x:c>
       <x:c r="H52" s="17" t="str">
-        <x:v>[4097,4098,4099,4100,4101,4102,4103,4104,4105,4106,4107,4108,4109,4110,4111,4112,4113,4114,4115,4116,4117,4118,4119,4120,4121,4122,4123]</x:v>
+        <x:v>[524417, 524546, 524675, 524804, 524933, 525062, 525191, 525320, 525449, 525578, 525707, 525836, 525965, 526094, 526223, 526352, 526481, 526610, 526739, 526868, 526997, 527126, 527255, 527384, 527513, 527642, 527771]</x:v>
       </x:c>
       <x:c r="I52" s="17" t="str">
-        <x:v>[4097,4098,4099,4100,4101,4102,4103,4104,4105,4106,4107,4108,4109,4110,4111,4112,4113,4114,4115,4116,4117,4118,4119,4120,4121,4122,4123]</x:v>
+        <x:v>[524417, 524546, 524675, 524804, 524933, 525062, 525191, 525320, 525449, 525578, 525707, 525836, 525965, 526094, 526223, 526352, 526481, 526610, 526739, 526868, 526997, 527126, 527255, 527384, 527513, 527642, 527771]</x:v>
       </x:c>
       <x:c r="J52" s="18" t="b">
         <x:v>1</x:v>
@@ -3617,13 +3617,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G53" s="17" t="str">
-        <x:v>[512,544,576,608,640,672,704,736,768,800,832,864,896,928,960,992,1024,1056,1088,1120,1152,1184,1216,1248,1280,1312]</x:v>
+        <x:v>[512, 544, 576, 608, 640, 672, 704, 736, 768, 800, 832, 864, 896, 928, 960, 992, 1024, 1056, 1088, 1120, 1152, 1184, 1216, 1248, 1280, 1312]</x:v>
       </x:c>
       <x:c r="H53" s="17" t="str">
-        <x:v>[1536,1632,1728,1824,1920,2016,2112,2208,2304,2400,2496,2592,2688,2784,2880,2976,3072,3168,3264,3360,3456,3552,3648,3744,3840,3936]</x:v>
+        <x:v>[196608, 208992, 221248, 233504, 245760, 258144, 270400, 282656, 294912, 307296, 319552, 331808, 344064, 356448, 368704, 380960, 393216, 405600, 417856, 430112, 442368, 454752, 467008, 479264, 491520, 503904]</x:v>
       </x:c>
       <x:c r="I53" s="17" t="str">
-        <x:v>[1536,1632,1728,1824,1920,2016,2112,2208,2304,2400,2496,2592,2688,2784,2880,2976,3072,3168,3264,3360,3456,3552,3648,3744,3840,3936]</x:v>
+        <x:v>[196608, 208992, 221248, 233504, 245760, 258144, 270400, 282656, 294912, 307296, 319552, 331808, 344064, 356448, 368704, 380960, 393216, 405600, 417856, 430112, 442368, 454752, 467008, 479264, 491520, 503904]</x:v>
       </x:c>
       <x:c r="J53" s="18" t="b">
         <x:v>0</x:v>
@@ -3677,13 +3677,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G54" s="17" t="str">
-        <x:v>[256,313,370,427,484,541,598,655,712,769,826,883,940,997,1054,1111,1168,1225,1282,1339,1396,1453,1510,1567,1624,1681,1738,1795]</x:v>
+        <x:v>[256, 313, 370, 427, 484, 541, 598, 655, 712, 769, 826, 883, 940, 997, 1054, 1111, 1168, 1225, 1282, 1339, 1396, 1453, 1510, 1567, 1624, 1681, 1738, 1795]</x:v>
       </x:c>
       <x:c r="H54" s="17" t="str">
-        <x:v>[2048,2139,2230,2321,2412,2503,2594,2685,2776,2867,2958,3049,3140,3231,3322,3413,3504,3595,3686,3777,3868,3959,4050,4141,4232,4323,4414,4505]</x:v>
+        <x:v>[262144, 273883, 285494, 297105, 308844, 320455, 332066, 343805, 355416, 367027, 378638, 390377, 401988, 413599, 425338, 436949, 448560, 460171, 471910, 483521, 495132, 506871, 518482, 530093, 541704, 553443, 565054, 576665]</x:v>
       </x:c>
       <x:c r="I54" s="17" t="str">
-        <x:v>[2048,2139,2230,2321,2412,2503,2594,2685,2776,2867,2958,3049,3140,3231,3322,3413,3504,3595,3686,3777,3868,3959,4050,4141,4232,4323,4414,4505]</x:v>
+        <x:v>[262144, 273883, 285494, 297105, 308844, 320455, 332066, 343805, 355416, 367027, 378638, 390377, 401988, 413599, 425338, 436949, 448560, 460171, 471910, 483521, 495132, 506871, 518482, 530093, 541704, 553443, 565054, 576665]</x:v>
       </x:c>
       <x:c r="J54" s="18" t="b">
         <x:v>1</x:v>
@@ -3737,13 +3737,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G55" s="17" t="str">
-        <x:v>[640,677,714,751,788,825,862,899,936,973,1010,1047,1084,1121,1158,1195,1232,1269,1306,1343,1380,1417,1454,1491,1528,1565,1602,1639,1676,1713]</x:v>
+        <x:v>[640, 677, 714, 751, 788, 825, 862, 899, 936, 973, 1010, 1047, 1084, 1121, 1158, 1195, 1232, 1269, 1306, 1343, 1380, 1417, 1454, 1491, 1528, 1565, 1602, 1639, 1676, 1713]</x:v>
       </x:c>
       <x:c r="H55" s="17" t="str">
-        <x:v>[3072,3155,3238,3321,3404,3487,3570,3653,3736,3819,3902,3985,4068,4151,4234,4317,4400,4483,4566,4649,4732,4815,4898,4981,5064,5147,5230,5313,5396,5479]</x:v>
+        <x:v>[3072, 3155, 3238, 3321, 3404, 3487, 3570, 3653, 3736, 3819, 3902, 3985, 4068, 4151, 4234, 4317, 4400, 4483, 4566, 4649, 4732, 4815, 4898, 4981, 5064, 5147, 5230, 5313, 5396, 5479]</x:v>
       </x:c>
       <x:c r="I55" s="17" t="str">
-        <x:v>[3072,3155,3238,3321,3404,3487,3570,3653,3736,3819,3902,3985,4068,4151,4234,4317,4400,4483,4566,4649,4732,4815,4898,4981,5064,5147,5230,5313,5396,5479]</x:v>
+        <x:v>[3072, 3155, 3238, 3321, 3404, 3487, 3570, 3653, 3736, 3819, 3902, 3985, 4068, 4151, 4234, 4317, 4400, 4483, 4566, 4649, 4732, 4815, 4898, 4981, 5064, 5147, 5230, 5313, 5396, 5479]</x:v>
       </x:c>
       <x:c r="J55" s="18" t="b">
         <x:v>0</x:v>
@@ -3857,13 +3857,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G57" s="17" t="str">
-        <x:v>[384,464,544,624,704,784,864,944,1024,1104,1184,1264,1344,1424,1504,1584,1664,1744]</x:v>
+        <x:v>[384, 464, 544, 624, 704, 784, 864, 944, 1024, 1104, 1184, 1264, 1344, 1424, 1504, 1584, 1664, 1744]</x:v>
       </x:c>
       <x:c r="H57" s="17" t="str">
-        <x:v>[8192,8320,8448,8576,8704,8832,8960,9088,9216,9344,9472,9600,9728,9856,9984,10112,10240,10368]</x:v>
+        <x:v>[8192, 8320, 8448, 8576, 8704, 8832, 8960, 9088, 9216, 9344, 9472, 9600, 9728, 9856, 9984, 10112, 10240, 10368]</x:v>
       </x:c>
       <x:c r="I57" s="17" t="str">
-        <x:v>[8192,8320,8448,8576,8704,8832,8960,9088,9216,9344,9472,9600,9728,9856,9984,10112,10240,10368]</x:v>
+        <x:v>[8192, 8320, 8448, 8576, 8704, 8832, 8960, 9088, 9216, 9344, 9472, 9600, 9728, 9856, 9984, 10112, 10240, 10368]</x:v>
       </x:c>
       <x:c r="J57" s="18" t="b">
         <x:v>1</x:v>
@@ -3917,13 +3917,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G58" s="21" t="str">
-        <x:v>[128,136,144,152,160,168,176,184,192,200,208,216,224,232,240,248,256,264,272,280,288,296,304,312,320,328,336,344,352,360,368,376,384,392,400,408,416]</x:v>
+        <x:v>[128, 136, 144, 152, 160, 168, 176, 184, 192, 200, 208, 216, 224, 232, 240, 248, 256, 264, 272, 280, 288, 296, 304, 312, 320, 328, 336, 344, 352, 360, 368, 376, 384, 392, 400, 408, 416]</x:v>
       </x:c>
       <x:c r="H58" s="21" t="str">
-        <x:v>[512,520,528,536,544,552,560,568,576,584,592,600,608,616,624,632,640,648,656,664,672,680,688,696,704,712,720,728,736,744,752,760,768,776,784,792,800]</x:v>
+        <x:v>[65536, 66568, 67600, 68632, 69664, 70696, 71728, 72760, 73792, 74824, 75856, 76888, 77920, 78952, 79984, 81016, 81920, 82952, 83984, 85016, 86048, 87080, 88112, 89144, 90176, 91208, 92240, 93272, 94304, 95336, 96368, 97400, 98304, 99336, 100368, 101400, 102432]</x:v>
       </x:c>
       <x:c r="I58" s="21" t="str">
-        <x:v>[512,520,528,536,544,552,560,568,576,584,592,600,608,616,624,632,640,648,656,664,672,680,688,696,704,712,720,728,736,744,752,760,768,776,784,792,800]</x:v>
+        <x:v>[65536, 66568, 67600, 68632, 69664, 70696, 71728, 72760, 73792, 74824, 75856, 76888, 77920, 78952, 79984, 81016, 81920, 82952, 83984, 85016, 86048, 87080, 88112, 89144, 90176, 91208, 92240, 93272, 94304, 95336, 96368, 97400, 98304, 99336, 100368, 101400, 102432]</x:v>
       </x:c>
       <x:c r="J58" s="22" t="b">
         <x:v>0</x:v>
@@ -3954,13 +3954,13 @@
       </x:c>
       <x:c r="S58" s="21" t="str"/>
       <x:c r="T58" s="23" t="str">
-        <x:v>SI_WB_060 batch37_noncausal_q64_kv4_small_varlen 覆盖: batch=37；q64/kv4；短序列多batch；非2次幂batch 设计: 用较小序列控制运行成本，同时覆盖高batch数量和q64/kv4组合。</x:v>
+        <x:v>SI_WB_060 batch37_noncausal_q64_kv4_small_varlen 覆盖: batch=37；q64/kv4；短query多batch；非2次幂batch 设计: 保持query较短控制输出规模，同时将KV/prompt提升到64K以上覆盖高batch长KV组合。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R534c94d593944078"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d8c35960dd74724"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Stabilize StemIndexer long KV pytest cases
</commit_message>
<xml_diff>
--- a/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
+++ b/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re6b79c4f76304a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R54419d1a98974023"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1068,9 +1068,11 @@
       <x:c r="R10" s="17" t="str">
         <x:v>FP32</x:v>
       </x:c>
-      <x:c r="S10" s="17" t="str"/>
+      <x:c r="S10" s="17" t="str">
+        <x:v>qflat=constant_positive; kflat=constant_positive; vbias=strictly_ascending_by_k_block</x:v>
+      </x:c>
       <x:c r="T10" s="19" t="str">
-        <x:v>SI_WB_009 causal_early_query_clip 覆盖: causal=true；early q block；s2Valid小于max_Kb；forced因果裁剪 设计: 早期 query 块只能看到历史块，验证因果路径不会选未来块。</x:v>
+        <x:v>SI_WB_009 causal_early_query_clip 覆盖: causal=true；early q block；s2Valid小于max_Kb；forced因果裁剪 设计: 早期 query 块只能看到历史块，并用确定性分数稳定长KV TopK边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -2028,9 +2030,11 @@
       <x:c r="R26" s="17" t="str">
         <x:v>FP32</x:v>
       </x:c>
-      <x:c r="S26" s="17" t="str"/>
+      <x:c r="S26" s="17" t="str">
+        <x:v>qflat=constant_positive; kflat=constant_positive; vbias=strictly_ascending_by_k_block</x:v>
+      </x:c>
       <x:c r="T26" s="19" t="str">
-        <x:v>SI_WB_025 gqa_q64_kv4_batch15_g16 覆盖: q_heads=64；kv_heads=4；g=16 设计: 覆盖 q_heads=64 与中间 kv_heads 组合。</x:v>
+        <x:v>SI_WB_025 gqa_q64_kv4_batch15_g16 覆盖: q_heads=64；kv_heads=4；g=16 设计: 覆盖 q_heads=64 与中间 kv_heads 组合，并用确定性分数稳定长KV TopK边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
@@ -2148,9 +2152,11 @@
       <x:c r="R28" s="17" t="str">
         <x:v>FP32</x:v>
       </x:c>
-      <x:c r="S28" s="17" t="str"/>
+      <x:c r="S28" s="17" t="str">
+        <x:v>qflat=constant_positive; kflat=constant_positive; vbias=strictly_ascending_by_k_block</x:v>
+      </x:c>
       <x:c r="T28" s="19" t="str">
-        <x:v>SI_WB_027 batch17_varlen_prefill_g16 覆盖: batch=17；变长q/kv；per-batch实际长度；prompt按batch实际长度输入 设计: 覆盖多 batch 负载不均；BNSD下q/kv seq_lens和num_prompt_tokens均按batch实际长度读取。</x:v>
+        <x:v>SI_WB_027 batch17_varlen_prefill_g16 覆盖: batch=17；变长q/kv；per-batch实际长度；prompt按batch实际长度输入 设计: 覆盖多 batch 负载不均，并用确定性分数稳定长KV TopK边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
@@ -3652,9 +3658,11 @@
       <x:c r="R53" s="17" t="str">
         <x:v>FP32</x:v>
       </x:c>
-      <x:c r="S53" s="17" t="str"/>
+      <x:c r="S53" s="17" t="str">
+        <x:v>qflat=constant_positive; kflat=constant_positive; vbias=strictly_ascending_by_k_block</x:v>
+      </x:c>
       <x:c r="T53" s="19" t="str">
-        <x:v>SI_WB_054 batch26_noncausal_q32_kv4_varlen 覆盖: batch=26；q32/kv4；non-causal；q尾块与kv尾块混合 设计: 补齐q32/kv4组合覆盖，验证中等GQA组下的多batch变长路径。</x:v>
+        <x:v>SI_WB_054 batch26_noncausal_q32_kv4_varlen 覆盖: batch=26；q32/kv4；non-causal；q尾块与kv尾块混合 设计: 补齐q32/kv4组合覆盖，并用确定性分数稳定长KV TopK边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
@@ -3960,7 +3968,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d8c35960dd74724"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6cfe200ceab454e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Revert "Stabilize StemIndexer long KV pytest cases"
This reverts commit a96ff5e07ca354989b44f635b2cdfb09111b927e.
</commit_message>
<xml_diff>
--- a/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
+++ b/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R54419d1a98974023"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re6b79c4f76304a16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1068,11 +1068,9 @@
       <x:c r="R10" s="17" t="str">
         <x:v>FP32</x:v>
       </x:c>
-      <x:c r="S10" s="17" t="str">
-        <x:v>qflat=constant_positive; kflat=constant_positive; vbias=strictly_ascending_by_k_block</x:v>
-      </x:c>
+      <x:c r="S10" s="17" t="str"/>
       <x:c r="T10" s="19" t="str">
-        <x:v>SI_WB_009 causal_early_query_clip 覆盖: causal=true；early q block；s2Valid小于max_Kb；forced因果裁剪 设计: 早期 query 块只能看到历史块，并用确定性分数稳定长KV TopK边界。</x:v>
+        <x:v>SI_WB_009 causal_early_query_clip 覆盖: causal=true；early q block；s2Valid小于max_Kb；forced因果裁剪 设计: 早期 query 块只能看到历史块，验证因果路径不会选未来块。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -2030,11 +2028,9 @@
       <x:c r="R26" s="17" t="str">
         <x:v>FP32</x:v>
       </x:c>
-      <x:c r="S26" s="17" t="str">
-        <x:v>qflat=constant_positive; kflat=constant_positive; vbias=strictly_ascending_by_k_block</x:v>
-      </x:c>
+      <x:c r="S26" s="17" t="str"/>
       <x:c r="T26" s="19" t="str">
-        <x:v>SI_WB_025 gqa_q64_kv4_batch15_g16 覆盖: q_heads=64；kv_heads=4；g=16 设计: 覆盖 q_heads=64 与中间 kv_heads 组合，并用确定性分数稳定长KV TopK边界。</x:v>
+        <x:v>SI_WB_025 gqa_q64_kv4_batch15_g16 覆盖: q_heads=64；kv_heads=4；g=16 设计: 覆盖 q_heads=64 与中间 kv_heads 组合。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
@@ -2152,11 +2148,9 @@
       <x:c r="R28" s="17" t="str">
         <x:v>FP32</x:v>
       </x:c>
-      <x:c r="S28" s="17" t="str">
-        <x:v>qflat=constant_positive; kflat=constant_positive; vbias=strictly_ascending_by_k_block</x:v>
-      </x:c>
+      <x:c r="S28" s="17" t="str"/>
       <x:c r="T28" s="19" t="str">
-        <x:v>SI_WB_027 batch17_varlen_prefill_g16 覆盖: batch=17；变长q/kv；per-batch实际长度；prompt按batch实际长度输入 设计: 覆盖多 batch 负载不均，并用确定性分数稳定长KV TopK边界。</x:v>
+        <x:v>SI_WB_027 batch17_varlen_prefill_g16 覆盖: batch=17；变长q/kv；per-batch实际长度；prompt按batch实际长度输入 设计: 覆盖多 batch 负载不均；BNSD下q/kv seq_lens和num_prompt_tokens均按batch实际长度读取。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
@@ -3658,11 +3652,9 @@
       <x:c r="R53" s="17" t="str">
         <x:v>FP32</x:v>
       </x:c>
-      <x:c r="S53" s="17" t="str">
-        <x:v>qflat=constant_positive; kflat=constant_positive; vbias=strictly_ascending_by_k_block</x:v>
-      </x:c>
+      <x:c r="S53" s="17" t="str"/>
       <x:c r="T53" s="19" t="str">
-        <x:v>SI_WB_054 batch26_noncausal_q32_kv4_varlen 覆盖: batch=26；q32/kv4；non-causal；q尾块与kv尾块混合 设计: 补齐q32/kv4组合覆盖，并用确定性分数稳定长KV TopK边界。</x:v>
+        <x:v>SI_WB_054 batch26_noncausal_q32_kv4_varlen 覆盖: batch=26；q32/kv4；non-causal；q尾块与kv尾块混合 设计: 补齐q32/kv4组合覆盖，验证中等GQA组下的多batch变长路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
@@ -3968,7 +3960,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6cfe200ceab454e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d8c35960dd74724"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine StemIndexer pytest case coverage
</commit_message>
<xml_diff>
--- a/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
+++ b/experimental/attention/stem_indexer/tests/pytest/excel/stem_indexer_cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R189f6a4830a242fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R3c1092de2b204779"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2451,7 +2451,7 @@
       </x:c>
       <x:c r="S35" s="9" t="str"/>
       <x:c r="T35" s="11" t="str">
-        <x:v>SI_WB_035 decode_prompt_128k_not_divisible 覆盖: decode；num_prompt_tokens非128整数倍；prompt block向上取整 设计: num_prompt_tokens=131071，验证128K附近promptLen向上取整路径。</x:v>
+        <x:v>SI_WB_034 decode_prompt_128k_not_divisible SI_WB_035 decode_prompt_128k_not_divisible 覆盖: decode；num_prompt_tokens非128整数倍；prompt block向上取整 设计: num_prompt_tokens=131071，验证128K附近promptLen向上取整路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2511,7 +2511,7 @@
       </x:c>
       <x:c r="S36" s="9" t="str"/>
       <x:c r="T36" s="11" t="str">
-        <x:v>SI_WB_036 dynamic_topk_small_upper_55 覆盖: 动态TopK small分支上边界；numPromptK=55 设计: prompt block数刚好小于56，验证kStart=numPromptK的边界。</x:v>
+        <x:v>SI_WB_035 dynamic_topk_small_upper_55 SI_WB_036 dynamic_topk_small_upper_55 覆盖: 动态TopK small分支上边界；numPromptK=55 设计: prompt block数刚好小于56，验证kStart=numPromptK的边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -2571,7 +2571,7 @@
       </x:c>
       <x:c r="S37" s="9" t="str"/>
       <x:c r="T37" s="11" t="str">
-        <x:v>SI_WB_037 dynamic_topk_medium_lower_56 覆盖: 动态TopK medium分支下边界；numPromptK=56 设计: prompt block数等于56，验证从small切到medium的分段点。</x:v>
+        <x:v>SI_WB_036 dynamic_topk_medium_lower_56 SI_WB_037 dynamic_topk_medium_lower_56 覆盖: 动态TopK medium分支下边界；numPromptK=56 设计: prompt block数等于56，验证从small切到medium的分段点。</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -2631,7 +2631,7 @@
       </x:c>
       <x:c r="S38" s="9" t="str"/>
       <x:c r="T38" s="11" t="str">
-        <x:v>SI_WB_038 dynamic_topk_medium_upper_159 覆盖: 动态TopK medium分支上边界；numPromptK=159；kv为32K token 设计: query长度保持不变，以32K KV覆盖medium分支高位边界。</x:v>
+        <x:v>SI_WB_037 dynamic_topk_medium_upper_159 SI_WB_038 dynamic_topk_medium_upper_159 覆盖: 动态TopK medium分支上边界；numPromptK=159；kv为32K token 设计: query长度保持不变，以32K KV覆盖medium分支高位边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2691,7 +2691,7 @@
       </x:c>
       <x:c r="S39" s="9" t="str"/>
       <x:c r="T39" s="11" t="str">
-        <x:v>SI_WB_039 dynamic_topk_large_lower_160 覆盖: 动态TopK large分支下边界；numPromptK=160；kv为32K token 设计: query长度保持不变，以32K KV覆盖从medium切到large的分段点。</x:v>
+        <x:v>SI_WB_038 dynamic_topk_large_lower_160 SI_WB_039 dynamic_topk_large_lower_160 覆盖: 动态TopK large分支下边界；numPromptK=160；kv为32K token 设计: query长度保持不变，以32K KV覆盖从medium切到large的分段点。</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2751,7 +2751,7 @@
       </x:c>
       <x:c r="S40" s="9" t="str"/>
       <x:c r="T40" s="11" t="str">
-        <x:v>SI_WB_040 batch12_mixed_prefill_decode 覆盖: batch=12；prefill/decode混合；多batch不同q/kv尾块 设计: 同一case内混合短prompt、q尾块、decode和kv尾块，验证batch维读取。</x:v>
+        <x:v>SI_WB_039 batch12_mixed_prefill_decode SI_WB_040 batch12_mixed_prefill_decode 覆盖: batch=12；prefill/decode混合；多batch不同q/kv尾块 设计: 同一case内混合短prompt、q尾块、decode和kv尾块，验证batch维读取。</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -2811,7 +2811,7 @@
       </x:c>
       <x:c r="S41" s="9" t="str"/>
       <x:c r="T41" s="11" t="str">
-        <x:v>SI_WB_041 causal_s1_s2_unequal_batch3_g16 覆盖: causal下S1/S2不相等；kbOffset参与dynamicTopK位置计算 设计: actS1=3、actS2=7，验证s1Pos和可见S2的偏移逻辑。</x:v>
+        <x:v>SI_WB_040 causal_s1_s2_unequal_batch3_g16 SI_WB_041 causal_s1_s2_unequal_batch3_g16 覆盖: causal下S1/S2不相等；kbOffset参与dynamicTopK位置计算 设计: actS1=3、actS2=7，验证s1Pos和可见S2的偏移逻辑。</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2871,7 +2871,7 @@
       </x:c>
       <x:c r="S42" s="9" t="str"/>
       <x:c r="T42" s="11" t="str">
-        <x:v>SI_WB_042 causal_q_tail_s1_s2_batch5 覆盖: causal；q尾块；S1/S2偏移；最后S1块可见范围变化 设计: q=385导致actS1=4，kv=1153导致actS2=10，同时覆盖尾块和因果偏移。</x:v>
+        <x:v>SI_WB_041 causal_q_tail_s1_s2_batch5 SI_WB_042 causal_q_tail_s1_s2_batch5 覆盖: causal；q尾块；S1/S2偏移；最后S1块可见范围变化 设计: q=385导致actS1=4，kv=1153导致actS2=10，同时覆盖尾块和因果偏移。</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2931,7 +2931,7 @@
       </x:c>
       <x:c r="S43" s="9" t="str"/>
       <x:c r="T43" s="11" t="str">
-        <x:v>SI_WB_043 gqa_q64_kv2_noncausal_s2_2048_blocks 覆盖: q_heads=64；kv_heads=2；g=32；non-causal；S2达到2048个block 设计: 组合大G和长S2，验证GQA映射和ProcessTopK多S2合并。</x:v>
+        <x:v>SI_WB_042 gqa_q64_kv2_noncausal_s2_2048_blocks SI_WB_043 gqa_q64_kv2_noncausal_s2_2048_blocks 覆盖: q_heads=64；kv_heads=2；g=32；non-causal；S2达到2048个block 设计: 组合大G和长S2，验证GQA映射和ProcessTopK多S2合并。</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -2991,7 +2991,7 @@
       </x:c>
       <x:c r="S44" s="9" t="str"/>
       <x:c r="T44" s="11" t="str">
-        <x:v>SI_WB_044 gqa_q64_kv8_m_tail 覆盖: q_heads=64；kv_heads=8；g=8；M方向尾块 设计: actS1=13时actS1*g=104，覆盖mBase=96后的尾块处理。</x:v>
+        <x:v>SI_WB_043 gqa_q64_kv8_m_tail SI_WB_044 gqa_q64_kv8_m_tail 覆盖: q_heads=64；kv_heads=8；g=8；M方向尾块 设计: actS1=13时actS1*g=104，覆盖mBase=96后的尾块处理。</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -3051,7 +3051,7 @@
       </x:c>
       <x:c r="S45" s="9" t="str"/>
       <x:c r="T45" s="11" t="str">
-        <x:v>SI_WB_045 short2_total_output_equal_batch4 覆盖: 短路2边界；curS2Len == initial + dynamicTopK + window 设计: prompt block=135，dynamicTopK=57，totalOutput=65，kv block=65，应直接输出连续索引。</x:v>
+        <x:v>SI_WB_044 short2_total_output_equal_batch4 SI_WB_045 short2_total_output_equal_batch4 覆盖: 短路2边界；curS2Len == initial + dynamicTopK + window 设计: prompt block=135，dynamicTopK=57，totalOutput=65，kv block=65，应直接输出连续索引。</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -3111,7 +3111,7 @@
       </x:c>
       <x:c r="S46" s="9" t="str"/>
       <x:c r="T46" s="11" t="str">
-        <x:v>SI_WB_046 short2_total_output_plus_one_batch4 覆盖: 短路2临界后一位；进入正常TopK路径 设计: prompt block=135，dynamicTopK=57，totalOutput=65，kv block=66，验证刚越过短路边界的行为。</x:v>
+        <x:v>SI_WB_045 short2_total_output_plus_one_batch4 SI_WB_046 short2_total_output_plus_one_batch4 覆盖: 短路2临界后一位；进入正常TopK路径 设计: prompt block=135，dynamicTopK=57，totalOutput=65，kv block=66，验证刚越过短路边界的行为。</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -3171,7 +3171,7 @@
       </x:c>
       <x:c r="S47" s="9" t="str"/>
       <x:c r="T47" s="11" t="str">
-        <x:v>SI_WB_047 batch23_noncausal_varlen_q32_kv8 覆盖: batch=23；non-causal；q/kv多batch变长；较大prompt block；q32/kv8 设计: 用非2次幂batch和递增长度组合，覆盖批量读取、shape最大值推导和non-causal全S2路径。</x:v>
+        <x:v>SI_WB_046 batch23_noncausal_varlen_q32_kv8 SI_WB_047 batch23_noncausal_varlen_q32_kv8 覆盖: batch=23；non-causal；q/kv多batch变长；较大prompt block；q32/kv8 设计: 用非2次幂batch和递增长度组合，覆盖批量读取、shape最大值推导和non-causal全S2路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -3231,7 +3231,7 @@
       </x:c>
       <x:c r="S48" s="9" t="str"/>
       <x:c r="T48" s="11" t="str">
-        <x:v>SI_WB_049 batch15_decode_prompt_tail_q64_kv4 覆盖: batch=15；decode；q=1；kv/prompt非128整数倍；q64/kv4 设计: 多batch decode同时覆盖prompt向上取整和不同KV尾块。</x:v>
+        <x:v>SI_WB_047 batch15_decode_prompt_tail_q64_kv4 SI_WB_049 batch15_decode_prompt_tail_q64_kv4 覆盖: batch=15；decode；q=1；kv/prompt非128整数倍；q64/kv4 设计: 多batch decode同时覆盖prompt向上取整和不同KV尾块。</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -3291,7 +3291,7 @@
       </x:c>
       <x:c r="S49" s="9" t="str"/>
       <x:c r="T49" s="11" t="str">
-        <x:v>SI_WB_050 batch4_dynamic_topk_boundary_mix 覆盖: 单case混合dynamicTopK边界55/56/159/160；batch=4；q64/kv8 设计: 将small/medium/large分段边界放在同一batch，验证每个batch独立读取prompt长度。</x:v>
+        <x:v>SI_WB_048 batch4_dynamic_topk_boundary_mix SI_WB_050 batch4_dynamic_topk_boundary_mix 覆盖: 单case混合dynamicTopK边界55/56/159/160；batch=4；q64/kv8 设计: 将small/medium/large分段边界放在同一batch，验证每个batch独立读取prompt长度。</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -3351,7 +3351,7 @@
       </x:c>
       <x:c r="S50" s="9" t="str"/>
       <x:c r="T50" s="11" t="str">
-        <x:v>SI_WB_051 batch24_noncausal_q32_kv2_varlen 覆盖: batch=24；q32/kv2；non-causal；多batch递增长度 设计: 补齐q32/kv2组合覆盖，验证较大batch下shape最大值推导和完整S2可见范围。</x:v>
+        <x:v>SI_WB_049 batch24_noncausal_q32_kv2_varlen SI_WB_051 batch24_noncausal_q32_kv2_varlen 覆盖: batch=24；q32/kv2；non-causal；多batch递增长度 设计: 补齐q32/kv2组合覆盖，验证较大batch下shape最大值推导和完整S2可见范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -3411,7 +3411,7 @@
       </x:c>
       <x:c r="S51" s="9" t="str"/>
       <x:c r="T51" s="11" t="str">
-        <x:v>SI_WB_052 batch25_causal_q32_kv2_tail_mix 覆盖: batch=25；q32/kv2；causal；q/kv均非128整数倍 设计: 用非整齐batch和尾块长度组合，验证causal下每个batch独立计算可见S2。</x:v>
+        <x:v>SI_WB_050 batch25_causal_q32_kv2_tail_mix SI_WB_052 batch25_causal_q32_kv2_tail_mix 覆盖: batch=25；q32/kv2；causal；q/kv均非128整数倍 设计: 用非整齐batch和尾块长度组合，验证causal下每个batch独立计算可见S2。</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -3471,7 +3471,7 @@
       </x:c>
       <x:c r="S52" s="9" t="str"/>
       <x:c r="T52" s="11" t="str">
-        <x:v>SI_WB_053 batch27_decode_q32_kv2_prompt_tail 覆盖: batch=27；q32/kv2；decode；prompt和kv均带尾块 设计: 多batch decode下验证num_prompt_tokens按batch读取，并覆盖prompt非128整数倍。</x:v>
+        <x:v>SI_WB_051 batch27_decode_q32_kv2_prompt_tail SI_WB_053 batch27_decode_q32_kv2_prompt_tail 覆盖: batch=27；q32/kv2；decode；prompt和kv均带尾块 设计: 多batch decode下验证num_prompt_tokens按batch读取，并覆盖prompt非128整数倍。</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -3531,7 +3531,7 @@
       </x:c>
       <x:c r="S53" s="9" t="str"/>
       <x:c r="T53" s="11" t="str">
-        <x:v>SI_WB_054 batch26_noncausal_q32_kv4_varlen 覆盖: batch=26；q32/kv4；non-causal；q尾块与kv尾块混合 设计: 补齐q32/kv4组合覆盖，验证中等GQA组下的多batch变长路径。</x:v>
+        <x:v>SI_WB_052 batch26_noncausal_q32_kv4_varlen SI_WB_054 batch26_noncausal_q32_kv4_varlen 覆盖: batch=26；q32/kv4；non-causal；q尾块与kv尾块混合 设计: 补齐q32/kv4组合覆盖，验证中等GQA组下的多batch变长路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3591,7 +3591,7 @@
       </x:c>
       <x:c r="S54" s="9" t="str"/>
       <x:c r="T54" s="11" t="str">
-        <x:v>SI_WB_055 batch28_causal_q32_kv4_offset_tail 覆盖: batch=28；q32/kv4；causal；S1/S2不等且均带尾块 设计: 通过非等差块边界长度覆盖causal可见范围偏移和尾块组合。</x:v>
+        <x:v>SI_WB_053 batch28_causal_q32_kv4_offset_tail SI_WB_055 batch28_causal_q32_kv4_offset_tail 覆盖: batch=28；q32/kv4；causal；S1/S2不等且均带尾块 设计: 通过非等差块边界长度覆盖causal可见范围偏移和尾块组合。</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -3651,7 +3651,7 @@
       </x:c>
       <x:c r="S55" s="9" t="str"/>
       <x:c r="T55" s="11" t="str">
-        <x:v>SI_WB_056 batch30_noncausal_q32_kv4_prompt_tail 覆盖: batch=30；q32/kv4；non-causal；prompt不能整除stem_block_size 设计: 大batch下每个batch的prompt长度不同，验证动态TopK预算读取不同prompt block。</x:v>
+        <x:v>SI_WB_054 batch30_noncausal_q32_kv4_prompt_tail SI_WB_056 batch30_noncausal_q32_kv4_prompt_tail 覆盖: batch=30；q32/kv4；non-causal；prompt不能整除stem_block_size 设计: 大batch下每个batch的prompt长度不同，验证动态TopK预算读取不同prompt block。</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -3711,7 +3711,7 @@
       </x:c>
       <x:c r="S56" s="9" t="str"/>
       <x:c r="T56" s="11" t="str">
-        <x:v>SI_WB_058 decode_q64_kv2_1m_tokens 覆盖: batch=1；q64/kv2；decode；KV长度达到1M token 设计: 大G decode路径下覆盖1M以内超长KV上限，验证prompt预算长度等于kv长度时的metadata和golden对齐。</x:v>
+        <x:v>SI_WB_055 decode_q64_kv2_1m_tokens SI_WB_058 decode_q64_kv2_1m_tokens 覆盖: batch=1；q64/kv2；decode；KV长度达到1M token 设计: 大G decode路径下覆盖1M以内超长KV上限，验证prompt预算长度等于kv长度时的metadata和golden对齐。</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -3771,7 +3771,7 @@
       </x:c>
       <x:c r="S57" s="9" t="str"/>
       <x:c r="T57" s="11" t="str">
-        <x:v>SI_WB_059 batch18_causal_q64_kv2_offset 覆盖: batch=18；q64/kv2；causal；S1/S2不等 设计: 最大GQA组下拉开q/kv块数，覆盖因果偏移和TPD衰减路径。</x:v>
+        <x:v>SI_WB_056 batch18_causal_q64_kv2_offset SI_WB_059 batch18_causal_q64_kv2_offset 覆盖: batch=18；q64/kv2；causal；S1/S2不等 设计: 最大GQA组下拉开q/kv块数，覆盖因果偏移和TPD衰减路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -3831,7 +3831,7 @@
       </x:c>
       <x:c r="S58" s="9" t="str"/>
       <x:c r="T58" s="11" t="str">
-        <x:v>SI_WB_060 batch37_noncausal_q64_kv4_small_varlen 覆盖: batch=37；q64/kv4；短query多batch；非2次幂batch 设计: 保持query较短控制输出规模，同时将KV/prompt提升到64K以上覆盖高batch长KV组合。</x:v>
+        <x:v>SI_WB_057 batch37_noncausal_q64_kv4_small_varlen SI_WB_060 batch37_noncausal_q64_kv4_small_varlen 覆盖: batch=37；q64/kv4；短query多batch；非2次幂batch 设计: 保持query较短控制输出规模，同时将KV/prompt提升到64K以上覆盖高batch长KV组合。</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -4919,34 +4919,34 @@
         <x:v>SI_WB_076</x:v>
       </x:c>
       <x:c r="B77" s="9" t="str">
-        <x:v>decode_q32_kv8_256k_prompt_512k</x:v>
+        <x:v>decode_long_kv_prompt_batch2</x:v>
       </x:c>
       <x:c r="C77" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D77" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E77" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F77" s="9" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="G77" s="11" t="str">
-        <x:v>[1]</x:v>
+        <x:v>[1,1]</x:v>
       </x:c>
       <x:c r="H77" s="11" t="str">
-        <x:v>[262144]</x:v>
+        <x:v>[262144,524288]</x:v>
       </x:c>
       <x:c r="I77" s="11" t="str">
-        <x:v>[524288]</x:v>
+        <x:v>[524288,1048576]</x:v>
       </x:c>
       <x:c r="J77" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K77" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="L77" s="9" t="n">
         <x:v>128</x:v>
@@ -4971,7 +4971,7 @@
       </x:c>
       <x:c r="S77" s="9" t="str"/>
       <x:c r="T77" s="11" t="str">
-        <x:v>SI_WB_076 decode_q32_kv8_256k_prompt_512k 覆盖: decode；KV=256K；prompt=512K 设计: 验证decode下prompt预算显著大于KV长度的路径。</x:v>
+        <x:v>SI_WB_076 decode_long_kv_prompt_batch2 覆盖: decode；KV=256K/512K；prompt=512K/1M；batch=2 设计: 将原两条长KV decode case合并到同一batch，验证prompt预算显著大于KV长度和large prompt分支。</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -4979,34 +4979,34 @@
         <x:v>SI_WB_077</x:v>
       </x:c>
       <x:c r="B78" s="9" t="str">
-        <x:v>decode_q64_kv4_512k_prompt_1m</x:v>
+        <x:v>causal_s2_512_1025_tail_batch2</x:v>
       </x:c>
       <x:c r="C78" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D78" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E78" s="9" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="F78" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G78" s="11" t="str">
-        <x:v>[1]</x:v>
+        <x:v>[1024,2048]</x:v>
       </x:c>
       <x:c r="H78" s="11" t="str">
-        <x:v>[524288]</x:v>
+        <x:v>[65536,131073]</x:v>
       </x:c>
       <x:c r="I78" s="11" t="str">
-        <x:v>[1048576]</x:v>
+        <x:v>[65536,131073]</x:v>
       </x:c>
       <x:c r="J78" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K78" s="9" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="L78" s="9" t="n">
         <x:v>128</x:v>
@@ -5031,7 +5031,7 @@
       </x:c>
       <x:c r="S78" s="9" t="str"/>
       <x:c r="T78" s="11" t="str">
-        <x:v>SI_WB_077 decode_q64_kv4_512k_prompt_1m 覆盖: decode；KV=512K；prompt=1M；q64/kv4 设计: 验证长KV decode和large prompt预算分支。</x:v>
+        <x:v>SI_WB_077 causal_s2_512_1025_tail_batch2 覆盖: causal；S2=512整块和1025 blocks尾块；batch=2 设计: 将S2长序列整块和尾块边界放入同一case，验证多S2 loop和因果可见范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -5039,31 +5039,31 @@
         <x:v>SI_WB_078</x:v>
       </x:c>
       <x:c r="B79" s="9" t="str">
-        <x:v>noncausal_q32_kv2_s2_512_blocks</x:v>
+        <x:v>causal_q32_kv4_q_gt_kv_small</x:v>
       </x:c>
       <x:c r="C79" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D79" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E79" s="9" t="n">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F79" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G79" s="11" t="str">
-        <x:v>[1024,2048]</x:v>
+        <x:v>[32768,16384,8192]</x:v>
       </x:c>
       <x:c r="H79" s="11" t="str">
-        <x:v>[65536,65536]</x:v>
+        <x:v>[8192,4096,2048]</x:v>
       </x:c>
       <x:c r="I79" s="11" t="str">
-        <x:v>[65536,65536]</x:v>
+        <x:v>[8192,4096,2048]</x:v>
       </x:c>
       <x:c r="J79" s="10" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K79" s="9" t="n">
         <x:v>1</x:v>
@@ -5091,7 +5091,7 @@
       </x:c>
       <x:c r="S79" s="9" t="str"/>
       <x:c r="T79" s="11" t="str">
-        <x:v>SI_WB_078 noncausal_q32_kv2_s2_512_blocks 覆盖: non-causal；S2=512 blocks；q32/kv2 设计: 覆盖S2分块大于两个baseN的整块路径。</x:v>
+        <x:v>SI_WB_078 causal_q32_kv4_q_gt_kv_small SI_WB_080 causal_q32_kv4_q_gt_kv_small 覆盖: causal；q_seq_lens大于kv_seq_lens；q32/kv4 设计: 覆盖Q长于KV时早期query不可见、后期query可见的裁剪路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -5099,34 +5099,34 @@
         <x:v>SI_WB_079</x:v>
       </x:c>
       <x:c r="B80" s="9" t="str">
-        <x:v>causal_q64_kv8_s2_1025_blocks_tail</x:v>
+        <x:v>noncausal_q64_kv2_q_gt_kv_tail</x:v>
       </x:c>
       <x:c r="C80" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D80" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E80" s="9" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="F80" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G80" s="11" t="str">
-        <x:v>[1024,2048]</x:v>
+        <x:v>[4097,8193,12289]</x:v>
       </x:c>
       <x:c r="H80" s="11" t="str">
-        <x:v>[131073,131073]</x:v>
+        <x:v>[2049,4097,6145]</x:v>
       </x:c>
       <x:c r="I80" s="11" t="str">
-        <x:v>[131073,131073]</x:v>
+        <x:v>[2049,4097,6145]</x:v>
       </x:c>
       <x:c r="J80" s="10" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K80" s="9" t="n">
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L80" s="9" t="n">
         <x:v>128</x:v>
@@ -5151,7 +5151,7 @@
       </x:c>
       <x:c r="S80" s="9" t="str"/>
       <x:c r="T80" s="11" t="str">
-        <x:v>SI_WB_079 causal_q64_kv8_s2_1025_blocks_tail 覆盖: causal；S2=1025 blocks带尾块；q64/kv8 设计: 覆盖长S2尾块和因果可见范围组合。</x:v>
+        <x:v>SI_WB_079 noncausal_q64_kv2_q_gt_kv_tail SI_WB_081 noncausal_q64_kv2_q_gt_kv_tail 覆盖: non-causal；q大于kv；q/kv均带尾块；q64/kv2 设计: 验证非因果路径下Q/KV长度大小关系不影响完整KV可见性。</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -5159,34 +5159,34 @@
         <x:v>SI_WB_080</x:v>
       </x:c>
       <x:c r="B81" s="9" t="str">
-        <x:v>causal_q32_kv4_q_gt_kv_small</x:v>
+        <x:v>alpha05_prompt_gt_kv_batch4</x:v>
       </x:c>
       <x:c r="C81" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D81" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E81" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F81" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G81" s="11" t="str">
-        <x:v>[32768,16384,8192]</x:v>
+        <x:v>[512,640,768,896]</x:v>
       </x:c>
       <x:c r="H81" s="11" t="str">
-        <x:v>[8192,4096,2048]</x:v>
+        <x:v>[32768,32768,65536,65536]</x:v>
       </x:c>
       <x:c r="I81" s="11" t="str">
-        <x:v>[8192,4096,2048]</x:v>
+        <x:v>[65536,98304,131072,196608]</x:v>
       </x:c>
       <x:c r="J81" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K81" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="L81" s="9" t="n">
         <x:v>128</x:v>
@@ -5211,7 +5211,7 @@
       </x:c>
       <x:c r="S81" s="9" t="str"/>
       <x:c r="T81" s="11" t="str">
-        <x:v>SI_WB_080 causal_q32_kv4_q_gt_kv_small 覆盖: causal；q_seq_lens大于kv_seq_lens；q32/kv4 设计: 覆盖Q长于KV时早期query不可见、后期query可见的裁剪路径。</x:v>
+        <x:v>SI_WB_080 alpha05_prompt_gt_kv_batch4 覆盖: alpha=0.5；prompt大于KV；prompt覆盖64K到192K；batch=4 设计: 合并prompt尺度和prompt&gt;KV预算场景，验证动态TopK预算按batch读取。</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -5219,7 +5219,7 @@
         <x:v>SI_WB_081</x:v>
       </x:c>
       <x:c r="B82" s="9" t="str">
-        <x:v>noncausal_q64_kv2_q_gt_kv_tail</x:v>
+        <x:v>dynamic_topk_small_medium_large_batch3</x:v>
       </x:c>
       <x:c r="C82" s="9" t="str">
         <x:v>PASS</x:v>
@@ -5231,22 +5231,22 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="F82" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G82" s="11" t="str">
-        <x:v>[4097,8193,12289]</x:v>
+        <x:v>[512,640,768]</x:v>
       </x:c>
       <x:c r="H82" s="11" t="str">
-        <x:v>[2049,4097,6145]</x:v>
+        <x:v>[7040,12800,25600]</x:v>
       </x:c>
       <x:c r="I82" s="11" t="str">
-        <x:v>[2049,4097,6145]</x:v>
+        <x:v>[7040,12800,25600]</x:v>
       </x:c>
       <x:c r="J82" s="10" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K82" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="L82" s="9" t="n">
         <x:v>128</x:v>
@@ -5271,7 +5271,7 @@
       </x:c>
       <x:c r="S82" s="9" t="str"/>
       <x:c r="T82" s="11" t="str">
-        <x:v>SI_WB_081 noncausal_q64_kv2_q_gt_kv_tail 覆盖: non-causal；q大于kv；q/kv均带尾块；q64/kv2 设计: 验证非因果路径下Q/KV长度大小关系不影响完整KV可见性。</x:v>
+        <x:v>SI_WB_081 dynamic_topk_small_medium_large_batch3 覆盖: dynamic TopK small/medium/large三段；prompt=55/100/200 blocks；batch=3 设计: 将原small、medium、large三条case合并，验证同一case内每个batch独立触发不同TopK预算分支。</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -5279,13 +5279,13 @@
         <x:v>SI_WB_082</x:v>
       </x:c>
       <x:c r="B83" s="9" t="str">
-        <x:v>alpha075_prompt_32k_to_128k_mix</x:v>
+        <x:v>s2_loop_255_256_257_batch3</x:v>
       </x:c>
       <x:c r="C83" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D83" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E83" s="9" t="n">
         <x:v>32</x:v>
@@ -5294,19 +5294,19 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G83" s="11" t="str">
-        <x:v>[512,640,768,896]</x:v>
+        <x:v>[512,512,512]</x:v>
       </x:c>
       <x:c r="H83" s="11" t="str">
-        <x:v>[32768,65536,98304,131072]</x:v>
+        <x:v>[32640,32768,32896]</x:v>
       </x:c>
       <x:c r="I83" s="11" t="str">
-        <x:v>[32768,65536,98304,131072]</x:v>
+        <x:v>[32640,32768,32896]</x:v>
       </x:c>
       <x:c r="J83" s="10" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K83" s="9" t="n">
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L83" s="9" t="n">
         <x:v>128</x:v>
@@ -5331,7 +5331,7 @@
       </x:c>
       <x:c r="S83" s="9" t="str"/>
       <x:c r="T83" s="11" t="str">
-        <x:v>SI_WB_082 alpha075_prompt_32k_to_128k_mix 覆盖: alpha=0.75；prompt覆盖32K到128K 设计: 覆盖TPD衰减中间值和多个prompt尺度。</x:v>
+        <x:v>SI_WB_082 s2_loop_255_256_257_batch3 SI_WB_087 s2_loop_255_256_257_batch3 覆盖: S2=255/256/257 blocks；baseN边界 设计: 验证S2 loop在整块边界前、正好边界、越过边界时的处理。</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -5339,13 +5339,13 @@
         <x:v>SI_WB_083</x:v>
       </x:c>
       <x:c r="B84" s="9" t="str">
-        <x:v>alpha05_prompt_gt_kv_noncausal</x:v>
+        <x:v>s2_loop_511_512_513_decode_batch3</x:v>
       </x:c>
       <x:c r="C84" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D84" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E84" s="9" t="n">
         <x:v>64</x:v>
@@ -5354,19 +5354,19 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G84" s="11" t="str">
-        <x:v>[512,640,768,896]</x:v>
+        <x:v>[1,1,1]</x:v>
       </x:c>
       <x:c r="H84" s="11" t="str">
-        <x:v>[32768,32768,32768,32768]</x:v>
+        <x:v>[65408,65536,65664]</x:v>
       </x:c>
       <x:c r="I84" s="11" t="str">
-        <x:v>[65536,98304,131072,196608]</x:v>
+        <x:v>[65408,65536,65664]</x:v>
       </x:c>
       <x:c r="J84" s="10" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K84" s="9" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L84" s="9" t="n">
         <x:v>128</x:v>
@@ -5391,7 +5391,7 @@
       </x:c>
       <x:c r="S84" s="9" t="str"/>
       <x:c r="T84" s="11" t="str">
-        <x:v>SI_WB_083 alpha05_prompt_gt_kv_noncausal 覆盖: alpha=0.5；non-causal；prompt大于KV 设计: 验证非因果路径下动态TopK预算仍按prompt变化。</x:v>
+        <x:v>SI_WB_083 s2_loop_511_512_513_decode_batch3 SI_WB_088 s2_loop_511_512_513_decode_batch3 覆盖: decode；S2=511/512/513 blocks 设计: 验证decode场景下多S2 loop边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -5399,13 +5399,13 @@
         <x:v>SI_WB_084</x:v>
       </x:c>
       <x:c r="B85" s="9" t="str">
-        <x:v>dynamic_topk_small_prompt_55_blocks_batch3</x:v>
+        <x:v>m_tail_g8_batch5</x:v>
       </x:c>
       <x:c r="C85" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D85" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E85" s="9" t="n">
         <x:v>32</x:v>
@@ -5414,16 +5414,16 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G85" s="11" t="str">
-        <x:v>[512,640,768]</x:v>
+        <x:v>[1536,1600,1664,1728,1792]</x:v>
       </x:c>
       <x:c r="H85" s="11" t="str">
-        <x:v>[7040,7040,7040]</x:v>
+        <x:v>[32768,33024,33280,33536,33792]</x:v>
       </x:c>
       <x:c r="I85" s="11" t="str">
-        <x:v>[7040,7040,7040]</x:v>
+        <x:v>[32768,33024,33280,33536,33792]</x:v>
       </x:c>
       <x:c r="J85" s="10" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K85" s="9" t="n">
         <x:v>1</x:v>
@@ -5451,7 +5451,7 @@
       </x:c>
       <x:c r="S85" s="9" t="str"/>
       <x:c r="T85" s="11" t="str">
-        <x:v>SI_WB_084 dynamic_topk_small_prompt_55_blocks_batch3 覆盖: prompt=55 blocks；dynamic TopK small分支上边界 设计: 补充small分支边界在多batch下的覆盖。</x:v>
+        <x:v>SI_WB_084 m_tail_g8_batch5 SI_WB_089 m_tail_g8_batch5 覆盖: gSize=8；M方向尾块；batch=5 设计: 覆盖GS1维度不能被mBase整除的尾块路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -5459,34 +5459,34 @@
         <x:v>SI_WB_085</x:v>
       </x:c>
       <x:c r="B86" s="9" t="str">
-        <x:v>dynamic_topk_medium_prompt_100_blocks_batch3</x:v>
+        <x:v>m_tail_g32_batch5</x:v>
       </x:c>
       <x:c r="C86" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D86" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E86" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F86" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G86" s="11" t="str">
-        <x:v>[512,640,768]</x:v>
+        <x:v>[384,512,640,768,896]</x:v>
       </x:c>
       <x:c r="H86" s="11" t="str">
-        <x:v>[12800,12928,13056]</x:v>
+        <x:v>[32768,33024,33280,33536,33792]</x:v>
       </x:c>
       <x:c r="I86" s="11" t="str">
-        <x:v>[12800,12928,13056]</x:v>
+        <x:v>[32768,33024,33280,33536,33792]</x:v>
       </x:c>
       <x:c r="J86" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K86" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="L86" s="9" t="n">
         <x:v>128</x:v>
@@ -5511,7 +5511,7 @@
       </x:c>
       <x:c r="S86" s="9" t="str"/>
       <x:c r="T86" s="11" t="str">
-        <x:v>SI_WB_085 dynamic_topk_medium_prompt_100_blocks_batch3 覆盖: prompt约100 blocks；dynamic TopK medium分支 设计: 覆盖medium分支的普通区间和轻微尾块。</x:v>
+        <x:v>SI_WB_085 m_tail_g32_batch5 SI_WB_090 m_tail_g32_batch5 覆盖: gSize=32；M方向尾块；batch=5 设计: 覆盖最大GQA组下的M分块尾块。</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -5519,34 +5519,34 @@
         <x:v>SI_WB_086</x:v>
       </x:c>
       <x:c r="B87" s="9" t="str">
-        <x:v>dynamic_topk_large_prompt_200_blocks_batch3</x:v>
+        <x:v>prompt_tail_gt_kv_batch6</x:v>
       </x:c>
       <x:c r="C87" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D87" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E87" s="9" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F87" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G87" s="11" t="str">
-        <x:v>[512,640,768]</x:v>
+        <x:v>[128,192,256,320,384,448]</x:v>
       </x:c>
       <x:c r="H87" s="11" t="str">
-        <x:v>[25600,25728,25856]</x:v>
+        <x:v>[32768,36864,40960,45056,49152,53248]</x:v>
       </x:c>
       <x:c r="I87" s="11" t="str">
-        <x:v>[25600,25728,25856]</x:v>
+        <x:v>[32769,36865,40961,45057,49153,53249]</x:v>
       </x:c>
       <x:c r="J87" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K87" s="9" t="n">
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L87" s="9" t="n">
         <x:v>128</x:v>
@@ -5571,7 +5571,7 @@
       </x:c>
       <x:c r="S87" s="9" t="str"/>
       <x:c r="T87" s="11" t="str">
-        <x:v>SI_WB_086 dynamic_topk_large_prompt_200_blocks_batch3 覆盖: prompt约200 blocks；dynamic TopK large分支 设计: 覆盖large分支和q64/kv4组合。</x:v>
+        <x:v>SI_WB_086 prompt_tail_gt_kv_batch6 SI_WB_091 prompt_tail_gt_kv_batch6 覆盖: prompt比KV多1 token；prompt尾块；batch=6 设计: 验证prompt ceil到block时的边界偏移。</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -5579,28 +5579,28 @@
         <x:v>SI_WB_087</x:v>
       </x:c>
       <x:c r="B88" s="9" t="str">
-        <x:v>s2_loop_255_256_257_batch3</x:v>
+        <x:v>kv_tail_1_token_batch7</x:v>
       </x:c>
       <x:c r="C88" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D88" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E88" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F88" s="9" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="G88" s="11" t="str">
-        <x:v>[512,512,512]</x:v>
+        <x:v>[256,320,384,448,512,576,640]</x:v>
       </x:c>
       <x:c r="H88" s="11" t="str">
-        <x:v>[32640,32768,32896]</x:v>
+        <x:v>[32769,40961,49153,57345,65537,73729,81921]</x:v>
       </x:c>
       <x:c r="I88" s="11" t="str">
-        <x:v>[32640,32768,32896]</x:v>
+        <x:v>[32769,40961,49153,57345,65537,73729,81921]</x:v>
       </x:c>
       <x:c r="J88" s="10" t="b">
         <x:v>0</x:v>
@@ -5631,7 +5631,7 @@
       </x:c>
       <x:c r="S88" s="9" t="str"/>
       <x:c r="T88" s="11" t="str">
-        <x:v>SI_WB_087 s2_loop_255_256_257_batch3 覆盖: S2=255/256/257 blocks；baseN边界 设计: 验证S2 loop在整块边界前、正好边界、越过边界时的处理。</x:v>
+        <x:v>SI_WB_087 kv_tail_1_token_batch7 SI_WB_092 kv_tail_1_token_batch7 覆盖: KV比整块多1 token；batch=7；q64/kv8 设计: 覆盖KV尾块最小非整块长度。</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -5639,28 +5639,28 @@
         <x:v>SI_WB_088</x:v>
       </x:c>
       <x:c r="B89" s="9" t="str">
-        <x:v>s2_loop_511_512_513_decode_batch3</x:v>
+        <x:v>q_tail_1_token_batch7</x:v>
       </x:c>
       <x:c r="C89" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D89" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E89" s="9" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F89" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G89" s="11" t="str">
-        <x:v>[1,1,1]</x:v>
+        <x:v>[129,257,385,513,641,769,897]</x:v>
       </x:c>
       <x:c r="H89" s="11" t="str">
-        <x:v>[65408,65536,65664]</x:v>
+        <x:v>[65536,66560,67584,68608,69632,70656,71680]</x:v>
       </x:c>
       <x:c r="I89" s="11" t="str">
-        <x:v>[65408,65536,65664]</x:v>
+        <x:v>[65536,66560,67584,68608,69632,70656,71680]</x:v>
       </x:c>
       <x:c r="J89" s="10" t="b">
         <x:v>1</x:v>
@@ -5691,7 +5691,7 @@
       </x:c>
       <x:c r="S89" s="9" t="str"/>
       <x:c r="T89" s="11" t="str">
-        <x:v>SI_WB_088 s2_loop_511_512_513_decode_batch3 覆盖: decode；S2=511/512/513 blocks 设计: 验证decode场景下多S2 loop边界。</x:v>
+        <x:v>SI_WB_088 q_tail_1_token_batch7 SI_WB_093 q_tail_1_token_batch7 覆盖: Q比整块多1 token；batch=7；q32/kv4 设计: 覆盖Q尾块最小非整块长度和causal偏移。</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -5699,34 +5699,34 @@
         <x:v>SI_WB_089</x:v>
       </x:c>
       <x:c r="B90" s="9" t="str">
-        <x:v>m_tail_g8_batch5</x:v>
+        <x:v>mixed_decode_prefill_q64_kv8_batch10</x:v>
       </x:c>
       <x:c r="C90" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D90" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E90" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F90" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G90" s="11" t="str">
-        <x:v>[1536,1600,1664,1728,1792]</x:v>
+        <x:v>[1,128,1,256,1,384,1,512,1,640]</x:v>
       </x:c>
       <x:c r="H90" s="11" t="str">
-        <x:v>[32768,33024,33280,33536,33792]</x:v>
+        <x:v>[32768,36864,40960,45056,49152,53248,57344,61440,65536,69632]</x:v>
       </x:c>
       <x:c r="I90" s="11" t="str">
-        <x:v>[32768,33024,33280,33536,33792]</x:v>
+        <x:v>[32768,36864,40960,45056,49152,53248,57344,61440,65536,69632]</x:v>
       </x:c>
       <x:c r="J90" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K90" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="L90" s="9" t="n">
         <x:v>128</x:v>
@@ -5751,7 +5751,7 @@
       </x:c>
       <x:c r="S90" s="9" t="str"/>
       <x:c r="T90" s="11" t="str">
-        <x:v>SI_WB_089 m_tail_g8_batch5 覆盖: gSize=8；M方向尾块；batch=5 设计: 覆盖GS1维度不能被mBase整除的尾块路径。</x:v>
+        <x:v>SI_WB_089 mixed_decode_prefill_q64_kv8_batch10 SI_WB_094 mixed_decode_prefill_q64_kv8_batch10 覆盖: decode/prefill交替；batch=10；q64/kv8 设计: 验证decode判定只依赖当前batch项，不影响同case内其他batch。</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -5759,34 +5759,34 @@
         <x:v>SI_WB_090</x:v>
       </x:c>
       <x:c r="B91" s="9" t="str">
-        <x:v>m_tail_g32_batch5</x:v>
+        <x:v>causal_offset_large_gap_batch6</x:v>
       </x:c>
       <x:c r="C91" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D91" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E91" s="9" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F91" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G91" s="11" t="str">
-        <x:v>[384,512,640,768,896]</x:v>
+        <x:v>[1024,1152,1280,1408,1536,1664]</x:v>
       </x:c>
       <x:c r="H91" s="11" t="str">
-        <x:v>[32768,33024,33280,33536,33792]</x:v>
+        <x:v>[262144,263168,264192,265216,266240,267264]</x:v>
       </x:c>
       <x:c r="I91" s="11" t="str">
-        <x:v>[32768,33024,33280,33536,33792]</x:v>
+        <x:v>[262144,263168,264192,265216,266240,267264]</x:v>
       </x:c>
       <x:c r="J91" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K91" s="9" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="L91" s="9" t="n">
         <x:v>128</x:v>
@@ -5811,7 +5811,7 @@
       </x:c>
       <x:c r="S91" s="9" t="str"/>
       <x:c r="T91" s="11" t="str">
-        <x:v>SI_WB_090 m_tail_g32_batch5 覆盖: gSize=32；M方向尾块；batch=5 设计: 覆盖最大GQA组下的M分块尾块。</x:v>
+        <x:v>SI_WB_090 causal_offset_large_gap_batch6 SI_WB_095 causal_offset_large_gap_batch6 覆盖: causal；S2远大于S1；256K级KV 设计: 覆盖大KV-Q偏移下的可见S2计算。</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -5819,31 +5819,31 @@
         <x:v>SI_WB_091</x:v>
       </x:c>
       <x:c r="B92" s="9" t="str">
-        <x:v>prompt_tail_gt_kv_batch6</x:v>
+        <x:v>noncausal_large_prompt_1m_qsmall</x:v>
       </x:c>
       <x:c r="C92" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D92" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E92" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F92" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G92" s="11" t="str">
-        <x:v>[128,192,256,320,384,448]</x:v>
+        <x:v>[128,256]</x:v>
       </x:c>
       <x:c r="H92" s="11" t="str">
-        <x:v>[32768,36864,40960,45056,49152,53248]</x:v>
+        <x:v>[131072,262144]</x:v>
       </x:c>
       <x:c r="I92" s="11" t="str">
-        <x:v>[32769,36865,40961,45057,49153,53249]</x:v>
+        <x:v>[1048576,1048576]</x:v>
       </x:c>
       <x:c r="J92" s="10" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K92" s="9" t="n">
         <x:v>1</x:v>
@@ -5871,7 +5871,7 @@
       </x:c>
       <x:c r="S92" s="9" t="str"/>
       <x:c r="T92" s="11" t="str">
-        <x:v>SI_WB_091 prompt_tail_gt_kv_batch6 覆盖: prompt比KV多1 token；prompt尾块；batch=6 设计: 验证prompt ceil到block时的边界偏移。</x:v>
+        <x:v>SI_WB_091 noncausal_large_prompt_1m_qsmall SI_WB_096 noncausal_large_prompt_1m_qsmall 覆盖: non-causal；prompt=1M；KV=128K/256K 设计: 验证large prompt预算上限和非因果完整KV可见路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -5879,34 +5879,34 @@
         <x:v>SI_WB_092</x:v>
       </x:c>
       <x:c r="B93" s="9" t="str">
-        <x:v>kv_tail_1_token_batch7</x:v>
+        <x:v>causal_prompt_256k_var_batch8</x:v>
       </x:c>
       <x:c r="C93" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D93" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E93" s="9" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F93" s="9" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="G93" s="11" t="str">
-        <x:v>[256,320,384,448,512,576,640]</x:v>
+        <x:v>[128,192,256,320,384,448,512,576]</x:v>
       </x:c>
       <x:c r="H93" s="11" t="str">
-        <x:v>[32769,40961,49153,57345,65537,73729,81921]</x:v>
+        <x:v>[262144,262656,263168,263680,264192,264704,265216,265728]</x:v>
       </x:c>
       <x:c r="I93" s="11" t="str">
-        <x:v>[32769,40961,49153,57345,65537,73729,81921]</x:v>
+        <x:v>[262144,262656,263168,263680,264192,264704,265216,265728]</x:v>
       </x:c>
       <x:c r="J93" s="10" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K93" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="L93" s="9" t="n">
         <x:v>128</x:v>
@@ -5931,7 +5931,7 @@
       </x:c>
       <x:c r="S93" s="9" t="str"/>
       <x:c r="T93" s="11" t="str">
-        <x:v>SI_WB_092 kv_tail_1_token_batch7 覆盖: KV比整块多1 token；batch=7；q64/kv8 设计: 覆盖KV尾块最小非整块长度。</x:v>
+        <x:v>SI_WB_092 causal_prompt_256k_var_batch8 SI_WB_097 causal_prompt_256k_var_batch8 覆盖: batch=8；256K级KV；causal；q32/kv8 设计: 覆盖中等batch下的长KV因果裁剪。</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -5939,34 +5939,34 @@
         <x:v>SI_WB_093</x:v>
       </x:c>
       <x:c r="B94" s="9" t="str">
-        <x:v>q_tail_1_token_batch7</x:v>
+        <x:v>causal_batch2_q64_kv8_exact_tail_blocks</x:v>
       </x:c>
       <x:c r="C94" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D94" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E94" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F94" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G94" s="11" t="str">
-        <x:v>[129,257,385,513,641,769,897]</x:v>
+        <x:v>[8192,8193]</x:v>
       </x:c>
       <x:c r="H94" s="11" t="str">
-        <x:v>[65536,66560,67584,68608,69632,70656,71680]</x:v>
+        <x:v>[32768,65537]</x:v>
       </x:c>
       <x:c r="I94" s="11" t="str">
-        <x:v>[65536,66560,67584,68608,69632,70656,71680]</x:v>
+        <x:v>[32768,65537]</x:v>
       </x:c>
       <x:c r="J94" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K94" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="L94" s="9" t="n">
         <x:v>128</x:v>
@@ -5991,7 +5991,7 @@
       </x:c>
       <x:c r="S94" s="9" t="str"/>
       <x:c r="T94" s="11" t="str">
-        <x:v>SI_WB_093 q_tail_1_token_batch7 覆盖: Q比整块多1 token；batch=7；q32/kv4 设计: 覆盖Q尾块最小非整块长度和causal偏移。</x:v>
+        <x:v>SI_WB_093 causal_batch2_q64_kv8_exact_tail_blocks 覆盖: causal；Q/KV整块和1 token尾块；q64/kv8；batch=2 设计: 将整块和尾块基线合并，验证长短两种块边界在同一case内处理正确。</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -5999,34 +5999,34 @@
         <x:v>SI_WB_094</x:v>
       </x:c>
       <x:c r="B95" s="9" t="str">
-        <x:v>mixed_decode_prefill_q64_kv8_batch10</x:v>
+        <x:v>noncausal_batch15_small_randomish_lengths</x:v>
       </x:c>
       <x:c r="C95" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D95" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E95" s="9" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F95" s="9" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="G95" s="11" t="str">
-        <x:v>[1,128,1,256,1,384,1,512,1,640]</x:v>
+        <x:v>[96,169,242,315,388,461,534,607,680,753,826,899,972,1045,1118]</x:v>
       </x:c>
       <x:c r="H95" s="11" t="str">
-        <x:v>[32768,36864,40960,45056,49152,53248,57344,61440,65536,69632]</x:v>
+        <x:v>[32768,34005,35242,36479,37716,38953,40190,41427,42664,43901,45138,46375,47612,48849,50086]</x:v>
       </x:c>
       <x:c r="I95" s="11" t="str">
-        <x:v>[32768,36864,40960,45056,49152,53248,57344,61440,65536,69632]</x:v>
+        <x:v>[32768,34069,35370,36671,37716,39017,40318,41619,42664,43965,45266,46567,47612,48913,50214]</x:v>
       </x:c>
       <x:c r="J95" s="10" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K95" s="9" t="n">
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L95" s="9" t="n">
         <x:v>128</x:v>
@@ -6051,7 +6051,7 @@
       </x:c>
       <x:c r="S95" s="9" t="str"/>
       <x:c r="T95" s="11" t="str">
-        <x:v>SI_WB_094 mixed_decode_prefill_q64_kv8_batch10 覆盖: decode/prefill交替；batch=10；q64/kv8 设计: 验证decode判定只依赖当前batch项，不影响同case内其他batch。</x:v>
+        <x:v>SI_WB_094 noncausal_batch15_small_randomish_lengths SI_WB_100 noncausal_batch15_small_randomish_lengths 覆盖: batch=15；不规则短query和KV尾块；non-causal 设计: 补充非规则长度泛化，避免只覆盖整齐等差长度。</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -6059,34 +6059,34 @@
         <x:v>SI_WB_095</x:v>
       </x:c>
       <x:c r="B96" s="9" t="str">
-        <x:v>causal_offset_large_gap_batch6</x:v>
+        <x:v>batch16_causal_varlen_q32_kv2</x:v>
       </x:c>
       <x:c r="C96" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D96" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E96" s="9" t="n">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F96" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G96" s="11" t="str">
-        <x:v>[1024,1152,1280,1408,1536,1664]</x:v>
+        <x:v>[138,276,404,542,642,769,896,1024,1153,1280,1408,1539,1678,1801,1965,2058]</x:v>
       </x:c>
       <x:c r="H96" s="11" t="str">
-        <x:v>[262144,263168,264192,265216,266240,267264]</x:v>
+        <x:v>[2048,4096,8195,12289,16384,32768,65536,45868,83231,98304,122880,131072,23421,167432,262144,204872]</x:v>
       </x:c>
       <x:c r="I96" s="11" t="str">
-        <x:v>[262144,263168,264192,265216,266240,267264]</x:v>
+        <x:v>[2048,4096,8195,12289,16384,32768,65536,45868,83231,98304,122880,131072,23421,167432,262144,204872]</x:v>
       </x:c>
       <x:c r="J96" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K96" s="9" t="n">
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L96" s="9" t="n">
         <x:v>128</x:v>
@@ -6111,7 +6111,7 @@
       </x:c>
       <x:c r="S96" s="9" t="str"/>
       <x:c r="T96" s="11" t="str">
-        <x:v>SI_WB_095 causal_offset_large_gap_batch6 覆盖: causal；S2远大于S1；256K级KV 设计: 覆盖大KV-Q偏移下的可见S2计算。</x:v>
+        <x:v>SI_WB_095 batch16_causal_varlen_q32_kv2 覆盖: batch=16；q32/kv2；causal；q/kv多batch变长；短KV、32K/64K/128K/256K混合 设计: 按SE补充的多batch变长规格覆盖metadata、shape推导、causal可见范围和prompt按batch读取。</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -6119,31 +6119,31 @@
         <x:v>SI_WB_096</x:v>
       </x:c>
       <x:c r="B97" s="9" t="str">
-        <x:v>noncausal_large_prompt_1m_qsmall</x:v>
+        <x:v>batch8_zero_len_causal_q32_kv8</x:v>
       </x:c>
       <x:c r="C97" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D97" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E97" s="9" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F97" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G97" s="11" t="str">
-        <x:v>[128,256]</x:v>
+        <x:v>[8192,0,8192,16384,65536,33489,2342,74523]</x:v>
       </x:c>
       <x:c r="H97" s="11" t="str">
-        <x:v>[131072,262144]</x:v>
+        <x:v>[2048,8192,0,8192,32768,66328,1234,3211]</x:v>
       </x:c>
       <x:c r="I97" s="11" t="str">
-        <x:v>[1048576,1048576]</x:v>
+        <x:v>[2048,8192,0,8192,32768,66328,1234,3211]</x:v>
       </x:c>
       <x:c r="J97" s="10" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K97" s="9" t="n">
         <x:v>1</x:v>
@@ -6171,7 +6171,7 @@
       </x:c>
       <x:c r="S97" s="9" t="str"/>
       <x:c r="T97" s="11" t="str">
-        <x:v>SI_WB_096 noncausal_large_prompt_1m_qsmall 覆盖: non-causal；prompt=1M；KV=128K/256K 设计: 验证large prompt预算上限和非因果完整KV可见路径。</x:v>
+        <x:v>SI_WB_096 batch8_zero_len_causal_q32_kv8 覆盖: batch=8；q32/kv8；causal；batch内混合q=0、kv=0、短KV和64K级KV 设计: 按SE补充的多batch零长度规格覆盖metadata、shape推导、空序列清理和causal可见范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -6179,34 +6179,34 @@
         <x:v>SI_WB_097</x:v>
       </x:c>
       <x:c r="B98" s="9" t="str">
-        <x:v>causal_prompt_256k_var_batch8</x:v>
+        <x:v>batch11_causal_q64_kv8_prompt_tail</x:v>
       </x:c>
       <x:c r="C98" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D98" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E98" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F98" s="9" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="G98" s="11" t="str">
-        <x:v>[128,192,256,320,384,448,512,576]</x:v>
+        <x:v>[257,385,513,641,769,897,1025,1153,1281,1409,1537]</x:v>
       </x:c>
       <x:c r="H98" s="11" t="str">
-        <x:v>[262144,262656,263168,263680,264192,264704,265216,265728]</x:v>
+        <x:v>[32768,49153,65536,81921,98304,114689,131072,147457,163840,180225,196608]</x:v>
       </x:c>
       <x:c r="I98" s="11" t="str">
-        <x:v>[262144,262656,263168,263680,264192,264704,265216,265728]</x:v>
+        <x:v>[32768,49281,65536,82049,98304,114817,131072,147585,163840,180353,196608]</x:v>
       </x:c>
       <x:c r="J98" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K98" s="9" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="L98" s="9" t="n">
         <x:v>128</x:v>
@@ -6231,7 +6231,7 @@
       </x:c>
       <x:c r="S98" s="9" t="str"/>
       <x:c r="T98" s="11" t="str">
-        <x:v>SI_WB_097 causal_prompt_256k_var_batch8 覆盖: batch=8；256K级KV；causal；q32/kv8 设计: 覆盖中等batch下的长KV因果裁剪。</x:v>
+        <x:v>SI_WB_097 batch11_causal_q64_kv8_prompt_tail 覆盖: batch=11；q64/kv8；causal；prompt大于KV且部分带尾块 设计: 补充较大batch下prompt预算与KV长度不同步增长的泛化组合。</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -6239,28 +6239,28 @@
         <x:v>SI_WB_098</x:v>
       </x:c>
       <x:c r="B99" s="9" t="str">
-        <x:v>noncausal_batch2_q64_kv8_exact_blocks</x:v>
+        <x:v>batch9_noncausal_q32_kv4_kv_scale_mix</x:v>
       </x:c>
       <x:c r="C99" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D99" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E99" s="9" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F99" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G99" s="11" t="str">
-        <x:v>[8192,16384]</x:v>
+        <x:v>[64,128,192,320,448,576,704,832,960]</x:v>
       </x:c>
       <x:c r="H99" s="11" t="str">
-        <x:v>[32768,65536]</x:v>
+        <x:v>[4096,8192,16384,32768,65536,98304,131072,196608,262144]</x:v>
       </x:c>
       <x:c r="I99" s="11" t="str">
-        <x:v>[32768,65536]</x:v>
+        <x:v>[4096,8192,16384,32768,65536,98304,131072,196608,262144]</x:v>
       </x:c>
       <x:c r="J99" s="10" t="b">
         <x:v>0</x:v>
@@ -6291,7 +6291,7 @@
       </x:c>
       <x:c r="S99" s="9" t="str"/>
       <x:c r="T99" s="11" t="str">
-        <x:v>SI_WB_098 noncausal_batch2_q64_kv8_exact_blocks 覆盖: non-causal；Q/KV均为整块；q64/kv8 设计: 作为较大整块输入的稳定基线。</x:v>
+        <x:v>SI_WB_098 batch9_noncausal_q32_kv4_kv_scale_mix 覆盖: batch=9；q32/kv4；non-causal；KV覆盖4K到256K多尺度 设计: 通过短query配合不同KV量级，验证non-causal完整S2路径和shape最大值推导。</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -6299,13 +6299,13 @@
         <x:v>SI_WB_099</x:v>
       </x:c>
       <x:c r="B100" s="9" t="str">
-        <x:v>causal_batch2_q64_kv2_tail_blocks</x:v>
+        <x:v>batch6_decode_prefill_q64_kv2_prompt_mix</x:v>
       </x:c>
       <x:c r="C100" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D100" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E100" s="9" t="n">
         <x:v>64</x:v>
@@ -6314,19 +6314,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G100" s="11" t="str">
-        <x:v>[8193,16385]</x:v>
+        <x:v>[1,128,1,256,1,512]</x:v>
       </x:c>
       <x:c r="H100" s="11" t="str">
-        <x:v>[32769,65537]</x:v>
+        <x:v>[65536,65536,131072,131072,262144,262144]</x:v>
       </x:c>
       <x:c r="I100" s="11" t="str">
-        <x:v>[32769,65537]</x:v>
+        <x:v>[65536,98304,131072,196608,262144,524288]</x:v>
       </x:c>
       <x:c r="J100" s="10" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K100" s="9" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="L100" s="9" t="n">
         <x:v>128</x:v>
@@ -6351,7 +6351,7 @@
       </x:c>
       <x:c r="S100" s="9" t="str"/>
       <x:c r="T100" s="11" t="str">
-        <x:v>SI_WB_099 causal_batch2_q64_kv2_tail_blocks 覆盖: causal；Q/KV均带1 token尾块；q64/kv2 设计: 覆盖最大gSize下Q/KV尾块叠加。</x:v>
+        <x:v>SI_WB_099 batch6_decode_prefill_q64_kv2_prompt_mix 覆盖: batch=6；q64/kv2；decode/prefill混合；prompt大于KV 设计: 同一case内交替decode和prefill，验证decode判断按batch生效且prompt预算独立读取。</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -6359,13 +6359,13 @@
         <x:v>SI_WB_100</x:v>
       </x:c>
       <x:c r="B101" s="9" t="str">
-        <x:v>noncausal_batch15_small_randomish_lengths</x:v>
+        <x:v>batch12_causal_q32_kv8_tail_scale_mix</x:v>
       </x:c>
       <x:c r="C101" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D101" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E101" s="9" t="n">
         <x:v>32</x:v>
@@ -6374,16 +6374,16 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G101" s="11" t="str">
-        <x:v>[96,169,242,315,388,461,534,607,680,753,826,899,972,1045,1118]</x:v>
+        <x:v>[129,257,386,514,643,771,900,1028,1157,1285,1414,1542]</x:v>
       </x:c>
       <x:c r="H101" s="11" t="str">
-        <x:v>[32768,34005,35242,36479,37716,38953,40190,41427,42664,43901,45138,46375,47612,48849,50086]</x:v>
+        <x:v>[2049,4097,8193,12289,16385,32769,49153,65537,98305,131073,196609,262145]</x:v>
       </x:c>
       <x:c r="I101" s="11" t="str">
-        <x:v>[32768,34069,35370,36671,37716,39017,40318,41619,42664,43965,45266,46567,47612,48913,50214]</x:v>
+        <x:v>[2049,4097,8193,12289,16385,32769,49153,65537,98305,131073,196609,262145]</x:v>
       </x:c>
       <x:c r="J101" s="10" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K101" s="9" t="n">
         <x:v>1</x:v>
@@ -6411,7 +6411,7 @@
       </x:c>
       <x:c r="S101" s="9" t="str"/>
       <x:c r="T101" s="11" t="str">
-        <x:v>SI_WB_100 noncausal_batch15_small_randomish_lengths 覆盖: batch=15；不规则短query和KV尾块；non-causal 设计: 补充非规则长度泛化，避免只覆盖整齐等差长度。</x:v>
+        <x:v>SI_WB_100 batch12_causal_q32_kv8_tail_scale_mix 覆盖: batch=12；q32/kv8；causal；Q/KV均带尾块且KV覆盖2K到256K 设计: 补充较多batch下尾块、长KV和causal偏移共同作用的泛化场景。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>